<commit_message>
fix: make logo background transparent (alpha)
</commit_message>
<xml_diff>
--- a/data/price.xlsx
+++ b/data/price.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Зручна таблиця" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Зручна таблиця" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O93"/>
+  <dimension ref="A1:O94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4999,6 +4999,75 @@
         </is>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>999999-TEST</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Тестовий товар</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>TEST_BRAND</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>100</v>
+      </c>
+      <c r="E94" t="n">
+        <v>90</v>
+      </c>
+      <c r="F94" t="n">
+        <v>10</v>
+      </c>
+      <c r="G94" t="n">
+        <v>5</v>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>50мл</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>TEST_COUNTRY</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Тестовий опис нот</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Объект испытания</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>Test item</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>Тестовое описание примечаний</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>Test description of notes</t>
+        </is>
+      </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>test.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore: sync price.xlsx and new product images
</commit_message>
<xml_diff>
--- a/data/price.xlsx
+++ b/data/price.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ПРОЕКТ AI\ЛИЧНЫЕ НАРАБОТКИ\AI Skin Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF242B31-3E9A-4895-9F11-BC1309E0508C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55CF0113-EC32-4FDB-875D-560D72D5D3F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1792" uniqueCount="790">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1861" uniqueCount="814">
   <si>
     <t>Артикул</t>
   </si>
@@ -3395,9 +3395,6 @@
 🌟 CEF Lab Intensive Retinol Serum – твій must-have для глибокого антивікового догляду та сяючої шкіри! 🌟</t>
   </si>
   <si>
-    <t>Ретинолова старт-сироватка Ceramide CEF Lab 30мл</t>
-  </si>
-  <si>
     <t>1403</t>
   </si>
   <si>
@@ -4329,6 +4326,292 @@
 Тип шкіри: Чутлива, суха, куперозна
 Країна виробництва: 🇺🇦 Україна
 🌟 Strengthening Day Cream SPF 20 – твій must-have для щоденного захисту та здорової шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>🌸 Інтенсивна зміцнювальна маска «Розкішна Магнолія» 50 мл 🌸
+✨ Маска з екстрактом магнолії – справжня розкіш для чутливої та схильної до почервоніння шкіри! Вона дарує комфорт, ніжність та силу, допомагаючи твоїй шкірі сяяти здоров’ям.
+💎 Основні переваги:
+🌿 Заспокоює реактивну та подразнену шкіру
+💖 Зміцнює судини та зменшує їхню реактивність
+🛡️ Відновлює захисний бар’єр шкіри
+💧 Глибоко зволожує та тонізує
+🌸 Сприяє загоєнню дрібних тріщин
+🔥 Показання: купероз, розацеа, судинна сітка, почервоніння, сухість та чутливість.
+🌟 Склад – твій секрет краси: MAXnolia, гамамеліс, рутин, кофеїн, екстракти імбиру, лакриці, алое, пептиди та інші активи для гармонії та сяйва.
+💚 Відчуй ніжність магнолії та подаруй своїй шкірі розкішний догляд!</t>
+  </si>
+  <si>
+    <t>805</t>
+  </si>
+  <si>
+    <t>803</t>
+  </si>
+  <si>
+    <t>✨ SOS Serum for Sensitive &amp; Couperose Skin – миттєве заспокоєння та зміцнення! ✨
+🌿 Потужна терапевтична дія:
+💧 Глибоко зволожує та відновлює бар’єр шкіри
+🌸 Знімає подразнення, свербіж та запалення
+💎 Зміцнює стінки судин і капілярів
+🛡️ Корегує прояви куперозу та розацеа
+🌟 Освітлює пігментацію та вирівнює тон
+⚡ Підвищує поріг чутливості шкіри
+💚 Результат – спокійна, рівна та доглянута шкіра без почервонінь!
+📌 Ключові активні компоненти:
+🌺 Екстракт кори магнолії – протизапальна дія, зменшення подразнень
+☀️ Токоферол (вітамін Е) – антиоксидантний захист
+🍇 Виноградна вода – тонізація та відновлення
+🌱 Рутин та пептиди – зміцнення судин та підвищення еластичності
+💧 Гіалуронова кислота – глибоке зволоження та комфорт
+📌 Показання до застосування:
+Купероз та розацеа
+Судинна сітка та почервоніння
+Реактивна та суха шкіра
+Приливний рум’янець
+Локальні запалення
+Порушення мікроциркуляції
+📌 Як застосовувати:  
+Нанеси невелику кількість сироватки на очищену шкіру обличчя. Використовуй щодня, особливо ввечері для інтенсивного відновлення.
+✔️ Характеристики продукту:
+Тип: Інтенсивна SOS-сироватка
+Об’єм: 50 мл
+Призначення: Зміцнення судин, зволоження, освітлення пігментації, зняття подразнень
+Тип шкіри: Чутлива, суха, куперозна
+Країна виробництва: 🇺🇦 Україна
+🌟 SOS Serum – твій must-have для миттєвого заспокоєння та здорової шкіри без куперозу! 🌟</t>
+  </si>
+  <si>
+    <t>Нейроседативна заспокійлива маска SOS-терапія 50 мл</t>
+  </si>
+  <si>
+    <t>Інтенсивна SOS сиворотка для куперозної шкіри 50 мл</t>
+  </si>
+  <si>
+    <t>Інтенсивна зміцнювальний маска "розкішна магнолія" 50 мл</t>
+  </si>
+  <si>
+    <t>806</t>
+  </si>
+  <si>
+    <t>✨ Neuro-SOS Calming Mask – миттєве заспокоєння та комфорт для чутливої шкіри! ✨
+🌿 Інноваційна формула з пептидним комплексом моментальної дії:
+💎 Зменшує нервову реакцію на зовнішні подразники
+🌸 Заспокоює нейрогенне запалення та почервоніння
+💧 Підвищує поріг толерантності шкіри
+🛡️ Зміцнює капіляри та зменшує реактивність
+🌟 Відновлює баланс і дарує відчуття комфорту
+💚 Результат – спокійна, рівна та доглянута шкіра вже після першого застосування!
+📌 Ключові активні компоненти:
+🌺 Екстракт кораліни, каштану та амбора – протизапальна та зміцнювальна дія
+🥥 Олії таману, Моної де Таїті та андіроба – живлення та відновлення бар’єру
+🌸 MAXnolia та олія сливових кісточок – антиоксидантний захист і заспокоєння
+🌿 Escin ß-Sitosterol Phtosome®, ескулін, рутин – зміцнення судинної системи
+💧 Бета-глюкан та пептиди (ацетил-тетрапептид-40, трипептид-8, гексапептид-1) – зволоження та відновлення
+⚡ PINOLUMIN PWD та CM-Naringenin-Chalcone – зменшення реактивності та подразнень
+📌 Показання до застосування:
+Почервоніння та роздратування
+Купероз та розацеа
+Судинна сітка та зірочки
+Приливний рум’янець
+Порушення мікроциркуляції
+Чутлива та суха шкіра
+✔️ Характеристики продукту:
+Тип: Заспокійлива нейроседативна маска
+Об’єм: 50 мл
+Призначення: Заспокоєння, зміцнення судин, зменшення реактивності, зволоження
+Тип шкіри: Чутлива, суха, куперозна
+Країна виробництва: 🇺🇦 Україна
+🌟 Neuro-SOS Mask – твій must-have для миттєвого заспокоєння та здорової шкіри без подразнень! 🌟</t>
+  </si>
+  <si>
+    <t>Зміцнювалиний 2х-фазний Тонер для чутливої та куперозної шкіри 250 мл</t>
+  </si>
+  <si>
+    <t>811</t>
+  </si>
+  <si>
+    <t>✨ Strengthening 2-Phase Toner – щоденний догляд для чутливої та куперозної шкіри! ✨
+🌿 Формула без спирту:
+💧 Швидко заспокоює подразнення та знімає почервоніння
+🌸 Зменшує набряки та відновлює бар’єр шкіри
+💎 Зміцнює судини та капіляри
+🛡️ Вирівнює тон та підтримує баланс мікробіому
+💚 Результат – свіжа, спокійна та доглянута шкіра щодня!
+📌 Ключові активні компоненти:
+🌱 Гідролізат гамамелісу + квіткова вода – заспокоює та звужує пори
+⚡ Есцин + кофеїн – покращують мікроциркуляцію та знімають набряки
+💧 Пантенол + бісаболол – зволоження та відновлення
+🌸 Ніацинамід – вирівнює тон шкіри
+🌿 Пребіотики – підтримують баланс мікробіому
+🌺 Екстракт камелії – додаткове заспокоєння
+📌 Переваги:
+Зміцнення судин та зменшення куперозу
+Усунення набряків та почервонінь
+Відновлення захисного бар’єру
+📌 Як застосовувати:  
+Перед використанням струсити. Нанести тонер на ватний диск та протерти обличчя вранці й ввечері після очищення.
+✔️ Характеристики продукту:
+Тип: Двофазний тонер для чутливої та куперозної шкіри
+Об’єм: 250 мл
+Призначення: Заспокоєння, зміцнення судин, зменшення почервонінь, відновлення бар’єру
+Тип шкіри: Чутлива, суха, куперозна
+Країна виробництва: 🇺🇦 Україна
+🌟 Strengthening 2-Phase Toner – твій must-have для щоденного комфорту та здорової шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>Міцелярний очищувальний крем-гель для чутливої, куперозної шкіри 250 мл</t>
+  </si>
+  <si>
+    <t>809</t>
+  </si>
+  <si>
+    <t>✨ Micellar Cleansing Cream-Gel – ніжне очищення та захист для чутливої шкіри! ✨
+🌿 Формула для щоденного комфорту:
+💧 Делікатно очищує та видаляє макіяж без подразнень
+🌸 Заспокоює та зменшує почервоніння
+💎 Зміцнює судини та підтримує мікроциркуляцію
+🛡️ Захищає від окислювального стресу
+🌟 Підтримує синтез колагену та покращує загальний стан шкіри
+💚 Результат – чиста, свіжа та доглянута шкіра без відчуття сухості!
+📌 Ключові активні компоненти:
+🌺 Водорозчинна арганова олія – м’яке очищення без порушення гідроліпідного балансу
+🌸 Екстракт магнолії (Maxnolia) – антиоксидантний захист та заспокоєння
+🌱 Пептид Skinasensyl – зменшення чутливості та реактивності
+☕ Кофеїн – стимуляція мікроциркуляції та тонус шкіри
+🌼 Екстракти женьшеню, ромашки та інші фітоекстракти – живлення та відновлення
+💧 Вітамін Е та гліцерин – зволоження та еластичність
+📌 Переваги:
+М’яке очищення та видалення макіяжу
+Заспокійлива дія та антиоксидантний захист
+Стимуляція синтезу колагену
+Підтримка природного балансу шкіри
+📌 Як застосовувати:  
+Нанеси невелику кількість крем-гелю на вологу шкіру, легко помасажуй та змий водою. Використовуй вранці та ввечері.
+✔️ Характеристики продукту:
+Бренд: Smart4Derma
+Тип: Міцелярний очищувальний крем-гель
+Об’єм: 250 мл
+Призначення: Очищення, заспокоєння, зміцнення судин, антиоксидантний захист
+Тип шкіри: Чутлива, суха, куперозна
+Країна виробництва: 🇺🇦 Україна
+🌟 Smart4Derma Micellar Cream-Gel – твій must-have для ніжного очищення та здорової шкіри щодня! 🌟</t>
+  </si>
+  <si>
+    <t>Вдосконалений денний крем SPF 30 - 50 мл</t>
+  </si>
+  <si>
+    <t>730</t>
+  </si>
+  <si>
+    <t>✨ Advanced Day Cream SPF 30 – інтелектуальний догляд та захист! ✨
+🌿 Високотехнологічна формула:
+☀️ Захист від UVA/UVB-променів завдяки SPF 30
+💎 Активізує природні процеси регенерації
+🌸 Стимулює утворення нових клітин
+💧 Відновлює пружність та еластичність
+🌟 Формує овал обличчя та розгладжує зморшки
+💚 Результат – сяюча, підтягнута та захищена шкіра щодня!
+📌 Показання до застосування:
+Фото- та хроностаріння
+Зморшки та тьмяний колір обличчя
+Гіперпігментація
+Знижений тонус шкіри
+Профілактика біостаріння
+Догляд після інвазивних процедур
+📌 Ключові активні компоненти:
+🌱 Комплекс UVA/UVB-фільтрів – захист від сонця
+🥥 Олії ши, кіноа, бабасу та макадамії – живлення та відновлення
+💧 X50 Hyalufiller та гіалуронат натрію – глибоке зволоження та заповнення зморшок
+🌸 Lipobelle Soyaglycone – стимуляція синтезу колагену
+⚡ X50 Photoglow Powder – сяйво та рівний тон
+🌿 Phytopresome та ПДРН – регенерація та ревіталізація
+🥕 Олія моркви та олія ему – антиоксидантний захист
+📌 Як застосовувати:  
+Нанеси крем на очищену шкіру обличчя щоранку. Рівномірно розподіли по всій поверхні, уникаючи зони навколо очей.
+✔️ Характеристики продукту:
+Тип: Денний крем для зрілої шкіри
+Об’єм: 50 мл
+Призначення: Захист SPF 30, омолодження, відновлення пружності, освітлення пігментації
+Тип шкіри: Зріла, суха, комбінована
+Країна виробництва: 🇺🇦 Україна
+🌟 Advanced Day Cream SPF 30 – твій must-have для щоденного захисту та молодої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>Ретинолова старт-сироватка Ceramide CEF Lab 30 мл</t>
+  </si>
+  <si>
+    <t>Вдосконалювальний Крем з ретинолом та церамідами 50 мл</t>
+  </si>
+  <si>
+    <t>✨ Advanced Retinol &amp; Ceramide Cream – нічний антивіковий догляд! ✨
+🌿 Передова формула:
+💎 Мікрокапсульований ретинол – контрольована нічна ексфоліація без подразнень
+🌸 Цераміди – відновлення епідермального бар’єру та захист від втрати вологи
+💧 Гіалуронат натрію – глибоке зволоження та еластичність
+🛡️ ПДРН та Lipobelle Soyaglycone – стимуляція регенерації та синтезу колагену
+🌟 Рослинні олії (камелії, макадамії, амли, Моной де Таїті) – живлення та антиоксидантний захист
+💚 Результат – пружна, гладка та сяюча шкіра щоранку!
+📌 Дія крему:
+Розгладжує статичні та мімічні зморшки
+Відновлює пружність та еластичність
+Покращує колір обличчя та коригує постакне
+Забезпечує оптимальне зволоження
+Зміцнює дерма-епідермальне сполучення
+📌 Показання до застосування:
+Фото- та хроностаріння
+Зморшки та знижений тонус
+Тьмяний колір та гіперпігментація
+Профілактика біостаріння
+Догляд після інвазивних процедур
+📌 Як застосовувати:  
+Нанеси крем на очищену шкіру обличчя ввечері перед сном. Використовуй регулярно для максимального ефекту.
+✔️ Характеристики продукту:
+Тип: Антивіковий нічний крем
+Об’єм: 50 мл
+Призначення: Омолодження, освітлення, зволоження, відновлення бар’єру
+Тип шкіри: Зріла, суха, комбінована
+Країна виробництва: 🇺🇦 Україна
+🌟 Advanced Retinol &amp; Ceramide Cream – твій must-have для молодої та сяючої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>731</t>
+  </si>
+  <si>
+    <t>Вдосконалювальний Пептидний крем для періорбітальної зони очей 30 мл</t>
+  </si>
+  <si>
+    <t>734</t>
+  </si>
+  <si>
+    <t>✨ Advanced Peptide Eye Cream – інноваційний догляд для зони навколо очей! ✨
+🌿 Високотехнологічна формула з технологією «рідких пептидів»:
+💎 Ефективно розгладжує тонкі лінії та зморшки
+🌸 Забезпечує миттєвий ліфтинг і моделювання контуру
+💧 Синхронізує природні процеси відновлення шкіри
+🛡️ Запобігає антиоксидантному стресу
+⚡ Потужні провідникові системи доставляють активні комплекси безпосередньо до клітин
+💚 Результат – сяючий, свіжий та молодий погляд!
+📌 Ключові активні компоненти:
+🌱 Декапептиди та олігопептиди – стимуляція синтезу колагену, омолодження
+💧 Гіалуронат натрію – глибоке зволоження та еластичність
+🥭 Олія манго та макадамії – живлення та відновлення бар’єру
+🌊 Екстракт фукуса – антиоксидантний захист та тонізація
+⚡ Аргирелін та нанопептиди – зменшення мімічних зморшок
+🌸 Shadownyl та Agefinity – освітлення та ревіталізація
+📌 Показання до застосування:
+Фото- та хроностаріння
+Зморшки та знижений тонус шкіри
+Гіперпігментація
+Профілактика біостаріння
+Догляд після інвазивних процедур
+📌 Як застосовувати:  
+Нанеси невелику кількість крему на чисту шкіру навколо очей. Використовуй щодня вранці та/або ввечері.
+✔️ Характеристики продукту:
+Тип: Пептидний крем для періорбітальної зони
+Об’єм: 30 мл
+Призначення: Ліфтинг, омолодження, освітлення, зволоження
+Тип шкіри: Чутлива, суха, зріла
+Країна виробництва: 🇺🇦 Україна
+🌟 Advanced Peptide Eye Cream – твій must-have для сяючого та молодого погляду! 🌟</t>
   </si>
 </sst>
 </file>
@@ -5396,10 +5679,10 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" s="12" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>710</v>
+        <v>807</v>
       </c>
       <c r="C20" s="8" t="s">
         <v>658</v>
@@ -5419,18 +5702,18 @@
         <v>657</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="K20" s="18" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" s="12" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="C21" s="8" t="s">
         <v>658</v>
@@ -5450,18 +5733,18 @@
         <v>657</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
       <c r="K21" s="18" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" s="12" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="C22" s="8" t="s">
         <v>658</v>
@@ -5481,18 +5764,18 @@
         <v>657</v>
       </c>
       <c r="J22" s="8" t="s">
+        <v>716</v>
+      </c>
+      <c r="K22" s="18" t="s">
         <v>717</v>
-      </c>
-      <c r="K22" s="18" t="s">
-        <v>718</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" s="12" t="s">
-        <v>721</v>
+        <v>720</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>719</v>
+        <v>718</v>
       </c>
       <c r="C23" s="8" t="s">
         <v>658</v>
@@ -5512,18 +5795,18 @@
         <v>657</v>
       </c>
       <c r="J23" s="8" t="s">
+        <v>719</v>
+      </c>
+      <c r="K23" s="18" t="s">
         <v>720</v>
-      </c>
-      <c r="K23" s="18" t="s">
-        <v>721</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" s="12" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="C24" s="8" t="s">
         <v>658</v>
@@ -5543,18 +5826,18 @@
         <v>657</v>
       </c>
       <c r="J24" s="8" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="K24" s="18" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" s="12" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="C25" s="8" t="s">
         <v>658</v>
@@ -5574,18 +5857,18 @@
         <v>657</v>
       </c>
       <c r="J25" s="8" t="s">
+        <v>725</v>
+      </c>
+      <c r="K25" s="18" t="s">
         <v>726</v>
-      </c>
-      <c r="K25" s="18" t="s">
-        <v>727</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" s="12" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="C26" s="8" t="s">
         <v>658</v>
@@ -5605,18 +5888,18 @@
         <v>657</v>
       </c>
       <c r="J26" s="8" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="K26" s="18" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" s="12" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="C27" s="8" t="s">
         <v>658</v>
@@ -5636,18 +5919,18 @@
         <v>657</v>
       </c>
       <c r="J27" s="8" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="K27" s="18" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" s="12" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="C28" s="8" t="s">
         <v>658</v>
@@ -5667,18 +5950,18 @@
         <v>657</v>
       </c>
       <c r="J28" s="8" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="K28" s="18" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" s="12" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="C29" s="8" t="s">
         <v>658</v>
@@ -5698,18 +5981,18 @@
         <v>657</v>
       </c>
       <c r="J29" s="8" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="K29" s="18" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" s="12" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="C30" s="8" t="s">
         <v>653</v>
@@ -5729,18 +6012,18 @@
         <v>657</v>
       </c>
       <c r="J30" s="8" t="s">
+        <v>740</v>
+      </c>
+      <c r="K30" s="18" t="s">
         <v>741</v>
-      </c>
-      <c r="K30" s="18" t="s">
-        <v>742</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" s="12" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="B31" s="8" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="C31" s="8" t="s">
         <v>653</v>
@@ -5760,18 +6043,18 @@
         <v>657</v>
       </c>
       <c r="J31" s="8" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="K31" s="18" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" s="12" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="B32" s="8" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="C32" s="8" t="s">
         <v>653</v>
@@ -5791,18 +6074,18 @@
         <v>657</v>
       </c>
       <c r="J32" s="8" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="K32" s="18" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" s="12" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="C33" s="8" t="s">
         <v>653</v>
@@ -5822,18 +6105,18 @@
         <v>657</v>
       </c>
       <c r="J33" s="8" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="K33" s="18" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" s="12" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="C34" s="8" t="s">
         <v>653</v>
@@ -5853,18 +6136,18 @@
         <v>657</v>
       </c>
       <c r="J34" s="8" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="K34" s="18" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" s="12" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="C35" s="8" t="s">
         <v>653</v>
@@ -5884,18 +6167,18 @@
         <v>657</v>
       </c>
       <c r="J35" s="8" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
       <c r="K35" s="18" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" s="12" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
       <c r="C36" s="8" t="s">
         <v>653</v>
@@ -5915,18 +6198,18 @@
         <v>657</v>
       </c>
       <c r="J36" s="8" t="s">
+        <v>759</v>
+      </c>
+      <c r="K36" s="18" t="s">
         <v>760</v>
-      </c>
-      <c r="K36" s="18" t="s">
-        <v>761</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" s="12" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>653</v>
@@ -5946,18 +6229,18 @@
         <v>657</v>
       </c>
       <c r="J37" s="8" t="s">
+        <v>762</v>
+      </c>
+      <c r="K37" s="18" t="s">
         <v>763</v>
-      </c>
-      <c r="K37" s="18" t="s">
-        <v>764</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" s="12" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="B38" s="8" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>653</v>
@@ -5977,18 +6260,18 @@
         <v>657</v>
       </c>
       <c r="J38" s="8" t="s">
+        <v>765</v>
+      </c>
+      <c r="K38" s="18" t="s">
         <v>766</v>
-      </c>
-      <c r="K38" s="18" t="s">
-        <v>767</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" s="12" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
       <c r="B39" s="8" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="C39" s="8" t="s">
         <v>653</v>
@@ -6008,18 +6291,18 @@
         <v>657</v>
       </c>
       <c r="J39" s="8" t="s">
-        <v>770</v>
+        <v>769</v>
       </c>
       <c r="K39" s="18" t="s">
-        <v>769</v>
+        <v>768</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" s="12" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
       <c r="B40" s="8" t="s">
-        <v>771</v>
+        <v>770</v>
       </c>
       <c r="C40" s="8" t="s">
         <v>653</v>
@@ -6039,18 +6322,18 @@
         <v>657</v>
       </c>
       <c r="J40" s="8" t="s">
-        <v>773</v>
+        <v>772</v>
       </c>
       <c r="K40" s="18" t="s">
-        <v>772</v>
+        <v>771</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" s="12" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
       <c r="B41" s="8" t="s">
-        <v>774</v>
+        <v>773</v>
       </c>
       <c r="C41" s="8" t="s">
         <v>653</v>
@@ -6070,18 +6353,18 @@
         <v>657</v>
       </c>
       <c r="J41" s="8" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="K41" s="18" t="s">
-        <v>775</v>
+        <v>774</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" s="12" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
       <c r="B42" s="8" t="s">
-        <v>777</v>
+        <v>776</v>
       </c>
       <c r="C42" s="8" t="s">
         <v>653</v>
@@ -6101,18 +6384,18 @@
         <v>657</v>
       </c>
       <c r="J42" s="8" t="s">
-        <v>779</v>
+        <v>778</v>
       </c>
       <c r="K42" s="18" t="s">
-        <v>778</v>
+        <v>777</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" s="12" t="s">
-        <v>782</v>
+        <v>781</v>
       </c>
       <c r="B43" s="8" t="s">
-        <v>780</v>
+        <v>779</v>
       </c>
       <c r="C43" s="8" t="s">
         <v>653</v>
@@ -6132,18 +6415,18 @@
         <v>657</v>
       </c>
       <c r="J43" s="8" t="s">
+        <v>780</v>
+      </c>
+      <c r="K43" s="18" t="s">
         <v>781</v>
-      </c>
-      <c r="K43" s="18" t="s">
-        <v>782</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" s="12" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
       <c r="B44" s="8" t="s">
-        <v>783</v>
+        <v>782</v>
       </c>
       <c r="C44" s="8" t="s">
         <v>653</v>
@@ -6157,24 +6440,24 @@
         <v>17</v>
       </c>
       <c r="H44" s="8" t="s">
-        <v>784</v>
+        <v>783</v>
       </c>
       <c r="I44" s="8" t="s">
         <v>657</v>
       </c>
       <c r="J44" s="8" t="s">
-        <v>786</v>
+        <v>785</v>
       </c>
       <c r="K44" s="18" t="s">
-        <v>785</v>
+        <v>784</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45" s="12" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
       <c r="B45" s="8" t="s">
-        <v>787</v>
+        <v>786</v>
       </c>
       <c r="C45" s="8" t="s">
         <v>653</v>
@@ -6194,227 +6477,395 @@
         <v>657</v>
       </c>
       <c r="J45" s="8" t="s">
-        <v>789</v>
+        <v>788</v>
       </c>
       <c r="K45" s="18" t="s">
-        <v>788</v>
+        <v>787</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A46" s="12"/>
-      <c r="B46" s="8"/>
+      <c r="A46" s="12" t="s">
+        <v>790</v>
+      </c>
+      <c r="B46" s="8" t="s">
+        <v>795</v>
+      </c>
       <c r="C46" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D46" s="8"/>
+      <c r="D46" s="8">
+        <v>640</v>
+      </c>
       <c r="E46" s="8"/>
       <c r="F46" s="8"/>
-      <c r="G46" s="8"/>
-      <c r="H46" s="8"/>
-      <c r="I46" s="8"/>
-      <c r="J46" s="8"/>
-      <c r="K46" s="18"/>
+      <c r="G46" s="8">
+        <v>29</v>
+      </c>
+      <c r="H46" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I46" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J46" s="8" t="s">
+        <v>789</v>
+      </c>
+      <c r="K46" s="18" t="s">
+        <v>790</v>
+      </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A47" s="12"/>
-      <c r="B47" s="8"/>
+      <c r="A47" s="12" t="s">
+        <v>791</v>
+      </c>
+      <c r="B47" s="8" t="s">
+        <v>794</v>
+      </c>
       <c r="C47" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D47" s="8"/>
+      <c r="D47" s="8">
+        <v>1460</v>
+      </c>
       <c r="E47" s="8"/>
       <c r="F47" s="8"/>
-      <c r="G47" s="8"/>
-      <c r="H47" s="8"/>
-      <c r="I47" s="8"/>
-      <c r="J47" s="8"/>
-      <c r="K47" s="18"/>
+      <c r="G47" s="8">
+        <v>17</v>
+      </c>
+      <c r="H47" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I47" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J47" s="8" t="s">
+        <v>792</v>
+      </c>
+      <c r="K47" s="18" t="s">
+        <v>791</v>
+      </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A48" s="12"/>
-      <c r="B48" s="8"/>
+      <c r="A48" s="12" t="s">
+        <v>796</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>793</v>
+      </c>
       <c r="C48" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D48" s="8"/>
+      <c r="D48" s="8">
+        <v>800</v>
+      </c>
       <c r="E48" s="8"/>
       <c r="F48" s="8"/>
-      <c r="G48" s="8"/>
-      <c r="H48" s="8"/>
-      <c r="I48" s="8"/>
-      <c r="J48" s="8"/>
-      <c r="K48" s="18"/>
+      <c r="G48" s="8">
+        <v>19</v>
+      </c>
+      <c r="H48" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I48" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J48" s="8" t="s">
+        <v>797</v>
+      </c>
+      <c r="K48" s="18" t="s">
+        <v>796</v>
+      </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A49" s="12"/>
-      <c r="B49" s="8"/>
+      <c r="A49" s="12" t="s">
+        <v>799</v>
+      </c>
+      <c r="B49" s="8" t="s">
+        <v>798</v>
+      </c>
       <c r="C49" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D49" s="8"/>
+      <c r="D49" s="8">
+        <v>860</v>
+      </c>
       <c r="E49" s="8"/>
       <c r="F49" s="8"/>
-      <c r="G49" s="8"/>
-      <c r="H49" s="8"/>
-      <c r="I49" s="8"/>
-      <c r="J49" s="8"/>
-      <c r="K49" s="18"/>
+      <c r="G49" s="8">
+        <v>22</v>
+      </c>
+      <c r="H49" s="8" t="s">
+        <v>672</v>
+      </c>
+      <c r="I49" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J49" s="8" t="s">
+        <v>800</v>
+      </c>
+      <c r="K49" s="18" t="s">
+        <v>799</v>
+      </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A50" s="12"/>
-      <c r="B50" s="9"/>
-      <c r="C50" s="9"/>
-      <c r="D50" s="8"/>
+      <c r="A50" s="12" t="s">
+        <v>802</v>
+      </c>
+      <c r="B50" s="8" t="s">
+        <v>801</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D50" s="8">
+        <v>800</v>
+      </c>
       <c r="E50" s="8"/>
       <c r="F50" s="8"/>
-      <c r="G50" s="8"/>
-      <c r="H50" s="8"/>
-      <c r="I50" s="8"/>
-      <c r="J50" s="9"/>
-      <c r="K50" s="15"/>
+      <c r="G50" s="8">
+        <v>25</v>
+      </c>
+      <c r="H50" s="8" t="s">
+        <v>672</v>
+      </c>
+      <c r="I50" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J50" s="8" t="s">
+        <v>803</v>
+      </c>
+      <c r="K50" s="18" t="s">
+        <v>802</v>
+      </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A51" s="12"/>
-      <c r="B51" s="9"/>
-      <c r="C51" s="9"/>
-      <c r="D51" s="8"/>
+      <c r="A51" s="12" t="s">
+        <v>805</v>
+      </c>
+      <c r="B51" s="8" t="s">
+        <v>804</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D51" s="8">
+        <v>1400</v>
+      </c>
       <c r="E51" s="8"/>
       <c r="F51" s="8"/>
-      <c r="G51" s="8"/>
-      <c r="H51" s="8"/>
-      <c r="I51" s="8"/>
-      <c r="J51" s="9"/>
-      <c r="K51" s="15"/>
+      <c r="G51" s="8">
+        <v>18</v>
+      </c>
+      <c r="H51" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I51" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J51" s="8" t="s">
+        <v>806</v>
+      </c>
+      <c r="K51" s="18" t="s">
+        <v>805</v>
+      </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A52" s="12"/>
-      <c r="B52" s="9"/>
-      <c r="C52" s="9"/>
-      <c r="D52" s="8"/>
+      <c r="A52" s="12" t="s">
+        <v>810</v>
+      </c>
+      <c r="B52" s="8" t="s">
+        <v>808</v>
+      </c>
+      <c r="C52" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D52" s="8">
+        <v>1260</v>
+      </c>
       <c r="E52" s="8"/>
       <c r="F52" s="8"/>
-      <c r="G52" s="8"/>
-      <c r="H52" s="8"/>
-      <c r="I52" s="8"/>
-      <c r="J52" s="9"/>
-      <c r="K52" s="15"/>
+      <c r="G52" s="8">
+        <v>26</v>
+      </c>
+      <c r="H52" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I52" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J52" s="8" t="s">
+        <v>809</v>
+      </c>
+      <c r="K52" s="18" t="s">
+        <v>810</v>
+      </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A53" s="12"/>
-      <c r="B53" s="9"/>
-      <c r="C53" s="9"/>
-      <c r="D53" s="8"/>
+      <c r="A53" s="12" t="s">
+        <v>812</v>
+      </c>
+      <c r="B53" s="8" t="s">
+        <v>811</v>
+      </c>
+      <c r="C53" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D53" s="8">
+        <v>800</v>
+      </c>
       <c r="E53" s="8"/>
       <c r="F53" s="8"/>
-      <c r="G53" s="8"/>
-      <c r="H53" s="8"/>
-      <c r="I53" s="8"/>
-      <c r="J53" s="9"/>
-      <c r="K53" s="15"/>
+      <c r="G53" s="8">
+        <v>24</v>
+      </c>
+      <c r="H53" s="8" t="s">
+        <v>664</v>
+      </c>
+      <c r="I53" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J53" s="8" t="s">
+        <v>813</v>
+      </c>
+      <c r="K53" s="18" t="s">
+        <v>812</v>
+      </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54" s="12"/>
-      <c r="B54" s="9"/>
-      <c r="C54" s="9"/>
+      <c r="B54" s="8"/>
+      <c r="C54" s="8" t="s">
+        <v>653</v>
+      </c>
       <c r="D54" s="8"/>
       <c r="E54" s="8"/>
       <c r="F54" s="8"/>
       <c r="G54" s="8"/>
       <c r="H54" s="8"/>
-      <c r="I54" s="8"/>
-      <c r="J54" s="9"/>
-      <c r="K54" s="15"/>
+      <c r="I54" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J54" s="8"/>
+      <c r="K54" s="18"/>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55" s="12"/>
-      <c r="B55" s="9"/>
-      <c r="C55" s="9"/>
+      <c r="B55" s="8"/>
+      <c r="C55" s="8" t="s">
+        <v>653</v>
+      </c>
       <c r="D55" s="8"/>
       <c r="E55" s="8"/>
       <c r="F55" s="8"/>
       <c r="G55" s="8"/>
       <c r="H55" s="8"/>
-      <c r="I55" s="8"/>
-      <c r="J55" s="9"/>
-      <c r="K55" s="15"/>
+      <c r="I55" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J55" s="8"/>
+      <c r="K55" s="18"/>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56" s="12"/>
-      <c r="B56" s="9"/>
-      <c r="C56" s="9"/>
+      <c r="B56" s="8"/>
+      <c r="C56" s="8" t="s">
+        <v>653</v>
+      </c>
       <c r="D56" s="8"/>
       <c r="E56" s="8"/>
       <c r="F56" s="8"/>
       <c r="G56" s="8"/>
       <c r="H56" s="8"/>
-      <c r="I56" s="8"/>
-      <c r="J56" s="9"/>
-      <c r="K56" s="15"/>
+      <c r="I56" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J56" s="8"/>
+      <c r="K56" s="18"/>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A57" s="12"/>
-      <c r="B57" s="9"/>
-      <c r="C57" s="9"/>
+      <c r="B57" s="8"/>
+      <c r="C57" s="8" t="s">
+        <v>653</v>
+      </c>
       <c r="D57" s="8"/>
       <c r="E57" s="8"/>
       <c r="F57" s="8"/>
       <c r="G57" s="8"/>
       <c r="H57" s="8"/>
-      <c r="I57" s="8"/>
-      <c r="J57" s="9"/>
-      <c r="K57" s="15"/>
+      <c r="I57" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J57" s="8"/>
+      <c r="K57" s="18"/>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A58" s="12"/>
-      <c r="B58" s="9"/>
-      <c r="C58" s="9"/>
+      <c r="B58" s="8"/>
+      <c r="C58" s="8" t="s">
+        <v>653</v>
+      </c>
       <c r="D58" s="8"/>
       <c r="E58" s="8"/>
       <c r="F58" s="8"/>
       <c r="G58" s="8"/>
       <c r="H58" s="8"/>
-      <c r="I58" s="8"/>
-      <c r="J58" s="9"/>
-      <c r="K58" s="15"/>
+      <c r="I58" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J58" s="8"/>
+      <c r="K58" s="18"/>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59" s="12"/>
-      <c r="B59" s="9"/>
-      <c r="C59" s="9"/>
+      <c r="B59" s="8"/>
+      <c r="C59" s="8" t="s">
+        <v>653</v>
+      </c>
       <c r="D59" s="8"/>
       <c r="E59" s="8"/>
       <c r="F59" s="8"/>
       <c r="G59" s="8"/>
       <c r="H59" s="8"/>
-      <c r="I59" s="8"/>
-      <c r="J59" s="9"/>
-      <c r="K59" s="15"/>
+      <c r="I59" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J59" s="8"/>
+      <c r="K59" s="18"/>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A60" s="12"/>
-      <c r="B60" s="9"/>
-      <c r="C60" s="9"/>
+      <c r="B60" s="8"/>
+      <c r="C60" s="8" t="s">
+        <v>653</v>
+      </c>
       <c r="D60" s="8"/>
       <c r="E60" s="8"/>
       <c r="F60" s="8"/>
       <c r="G60" s="8"/>
       <c r="H60" s="8"/>
-      <c r="I60" s="8"/>
-      <c r="J60" s="9"/>
-      <c r="K60" s="15"/>
+      <c r="I60" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J60" s="8"/>
+      <c r="K60" s="18"/>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A61" s="12"/>
-      <c r="B61" s="9"/>
-      <c r="C61" s="9"/>
+      <c r="B61" s="8"/>
+      <c r="C61" s="8" t="s">
+        <v>653</v>
+      </c>
       <c r="D61" s="8"/>
       <c r="E61" s="8"/>
       <c r="F61" s="8"/>
       <c r="G61" s="8"/>
       <c r="H61" s="8"/>
-      <c r="I61" s="8"/>
-      <c r="J61" s="9"/>
-      <c r="K61" s="15"/>
+      <c r="I61" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J61" s="8"/>
+      <c r="K61" s="18"/>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A62" s="12"/>
@@ -6425,7 +6876,9 @@
       <c r="F62" s="8"/>
       <c r="G62" s="8"/>
       <c r="H62" s="8"/>
-      <c r="I62" s="8"/>
+      <c r="I62" s="8" t="s">
+        <v>657</v>
+      </c>
       <c r="J62" s="9"/>
       <c r="K62" s="15"/>
     </row>

</xml_diff>

<commit_message>
feat: default theme dark on first visit
</commit_message>
<xml_diff>
--- a/data/price.xlsx
+++ b/data/price.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ПРОЕКТ AI\ЛИЧНЫЕ НАРАБОТКИ\AI Skin Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD4CE5F5-3CD7-4334-9485-B5DE7A3D7A0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98587DFA-14EC-468C-B9CD-64BE232C5C74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1922" uniqueCount="841">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2041" uniqueCount="899">
   <si>
     <t>Артикул</t>
   </si>
@@ -4946,6 +4946,644 @@
 Бренд: SMART DERMA
 Країна виробництва: 🇺🇦 Україна
 🌟 Arabica Coffee Eye Mask – твій must-have для сяючого та молодого погляду без темних кіл і набряків! 🌟</t>
+  </si>
+  <si>
+    <t>Інтелектуальна сироватка-елексир "БІОПЛАЗМА" з мультипептидами - 50 мл</t>
+  </si>
+  <si>
+    <t>✨ Bioplasma Peptide Elixir – концентрований інтелектуальний догляд! ✨
+🌿 Високотехнологічна формула для комплексного омолодження:
+💎 Відновлює пружність та еластичність завдяки комплексу пептидів
+💧 Забезпечує глибоке зволоження гіалуроновою кислотою
+🌸 Омега-насичена лляна олія живить та розгладжує
+🛡️ Активізує регенераційні процеси та захищає від стресу
+🌟 Дарує шкірі гладкість, сяйво та молодість
+💚 Результат – тонкі лінії та зморшки розгладжуються, шкіра виглядає здоровою та оновленою!
+📌 Ключові активні компоненти:
+🌱 Bioplasma™ FA та комплекс пептидів (Replexium, CAPS2GO™, Argireline, Agefinity™) – стимуляція синтезу колагену та регенерація
+💧 Гіалуронат натрію, Hyalurosmooth PW LS 8997, Hydagen® Aquaporin – глибоке зволоження та підтримка водного балансу
+🥥 Лляна олія, масла ши та авокадо – живлення та відновлення бар’єру
+🌸 Антарктицин, Easyliance, біотин трипептид-1 – ревіталізація та зміцнення шкіри
+⚡ Ацетил тетрапептид-2, ацетил гексапептид-1, олігопептиди та поліпептиди – омолодження та корекція зморшок
+📌 Показання до застосування:
+Щоденний догляд для уповільнення старіння
+Запобігання зморшкам
+Фото- та хроностаріння
+Тьмяний колір обличчя
+Гіперпігментація та знижений тонус
+Догляд після інвазивних процедур
+Вікова шкіра
+📌 Як застосовувати:  
+Нанеси кілька крапель еліксиру на очищену шкіру обличчя та шиї. Використовуй щодня для максимального ефекту омолодження.
+✔️ Характеристики продукту:
+Тип: Інтелектуальна антивікова сироватка-еліксир
+Об’єм: 50 мл
+Призначення: Омолодження, зволоження, відновлення, живлення
+Тип шкіри: Зріла, суха, комбінована
+Країна виробництва: 🇺🇦 Україна
+🌟 Bioplasma Peptide Elixir – твій must-have для молодої та сяючої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>704</t>
+  </si>
+  <si>
+    <t>Інтелектуального заповнювального Гідромісту – 250 мл</t>
+  </si>
+  <si>
+    <t>✨ Intelligent HydroMist – багатофункціональне зволоження та anti-age догляд! ✨
+🌿 Інноваційна формула для щоденного відновлення:
+💧 Миттєве та пролонговане зволоження
+🌸 Нормалізація pH та вирівнювання тону шкіри
+💎 Зменшення глибини зморшок та профілактика їх появи
+🛡️ Захист від сухості та еритеми
+🌟 Ефект сяйва зсередини
+💚 Результат – свіжа, гладка та сяюча шкіра щодня!
+📌 Ключові активні компоненти:
+❄️ Antarcticine® – морський інгредієнт із криопротекторними властивостями
+💧 Гіалуронат натрію та Hydagen® Aquaporin – глибоке зволоження та підтримка водного балансу
+🌱 SPAR'AGE™ та морські мінерали – ревіталізація та захист
+🌸 Амінокислоти та пантенол – живлення, відновлення та зміцнення шкіри
+📌 Показання до застосування:
+Щоденний догляд за віковою шкірою
+Профілактика старіння
+Відновлення після косметологічних процедур
+Борьба з гіперпігментацією та зниженим тонусом
+✔️ Характеристики продукту:
+Тип: Інтелектуальний заповнювальний гідроміст
+Об’єм: 250 мл
+Призначення: Зволоження, омолодження, захист, сяйво
+Тип шкіри: Всі типи, особливо суха та зріла
+Країна виробництва: 🇺🇦 Україна
+🌟 Intelligent HydroMist – твій must-have для миттєвого зволоження та сяючої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>703</t>
+  </si>
+  <si>
+    <t>Гель для вмивання "Активатор Енергії" з кислотами - 250 мл</t>
+  </si>
+  <si>
+    <t>✨ Energy Activator Cleansing Gel – перезарядка для твоєї шкіри! ✨
+🌿 Інноваційна формула з кислотами та ензимами:
+⚡ Перезаряджає клітини шкіри на 27%
+💧 Відновлює pH-баланс та підтримує оптимальний рівень зволоження
+🌸 Комплекс із трьох кислот у розчині електролітів – м’яке, але ефективне очищення
+🛡️ Компонент OXY 229 PF активує мітохондріальне дихання для енергії клітин
+💎 Дарує свіжість, сяйво та рівний тон
+💚 Результат – чиста, енергійна та сяюча шкіра після кожного вмивання!
+📌 Ключові активні компоненти:
+🌱 Гліколева, піруватна та ферулова кислоти – ексфоліація та вирівнювання тону
+⚡ OXY 229 PF – активація клітинної енергії
+💧 Гіалуронат натрію, сечовина, Д-пантенол – глибоке зволоження та відновлення
+🌸 Екстракт гібіскуса, морські мінерали – антиоксидантний захист та тонізація
+🌟 Hydagen® Aquaporin, Lys'lastine™ V, Perlaura® – підтримка водного балансу та пружності
+📌 Показання до застосування:
+Уповільнення старіння без радикальних методів
+Запобігання появі зморшок
+Фото- та хроностаріння
+Тьмяний колір обличчя
+Гіперпігментація
+Знижений тонус шкіри
+Догляд після інвазивних процедур
+📌 Як застосовувати:  
+Нанеси невелику кількість гелю на вологу шкіру, розподіли по масажних лініях, легко промасажуй та змий теплою водою. Використовуй щодня для максимального ефекту.
+✔️ Характеристики продукту:
+Тип: Інноваційний гель для вмивання
+Об’єм: 250 мл
+Призначення: Очищення, омолодження, відновлення енергії клітин
+Тип шкіри: Вікова, комбінована, проблемна
+Країна виробництва: 🇺🇦 Україна
+🌟 Energy Activator Cleansing Gel – твій must-have для щоденного енергетичного догляду! 🌟</t>
+  </si>
+  <si>
+    <t>700</t>
+  </si>
+  <si>
+    <t>SMART4DERMA Aquagen - Двоетапна система інтенсивного зволоження 2х75</t>
+  </si>
+  <si>
+    <t>2х75 мл</t>
+  </si>
+  <si>
+    <t>✨ SMART4DERMA Aquagen – інноваційна система догляду з урахуванням циркадних ритмів! ✨
+🌿 Двоетапна формула для глибокого зволоження, живлення та ревіталізації:
+💧 Відновлює баланс вологи та мікробіом шкіри
+🌸 Стимулює синтез колагену та забезпечує ліфтинг
+💎 Освітлює пігментацію та повертає природне сяйво
+🛡️ Захищає від зовнішніх факторів та фотостаріння
+💚 Результат – пружна, сяюча та здорова шкіра з ефектом перетворення!
+📌 Система включає дві маски:
+1️⃣ 4D Aqua Mask Vita C &amp; Probiotic (75 мл)
+Збагачена вітамінами та пребіотиками
+Містить чотири види гіалуронової кислоти
+Відновлює мікробіом, покращує тон та тургор
+Захищає від зовнішніх факторів
+2️⃣ Bakuchiol Mask Ceramides &amp; AA2G (75 мл)
+Глибоко зволожує та оздоровлює шкіру
+Розгладжує зморшки та освітлює пігментацію
+Повертає природне сяйво та еластичність
+📌 Активні інгредієнти:
+🌱 Крок 1: Сік алое, Hydagen® Aquaporin, 4D гіалуронова кислота, пребіотики, Д-пантенол, вітаміни В3 і С, кофеїн, біотин, Amitose 3GA
+🌸 Крок 2: Олії ши та оливки, бакухіол, сквалан, BIO CERAMIDYL PURE, гідролізовані протеїни пшениці, вівса, шовку та рису
+✔️ Характеристики продукту:
+Тип: Двоетапна система інтенсивного зволоження
+Об’єм: 2×75 мл
+Призначення: Зволоження, живлення, ліфтинг, освітлення
+Тип шкіри: Всі типи, особливо суха та зріла
+Бренд: SMART4DERMA
+Країна виробництва: 🇺🇦 Україна
+🌟 SMART4DERMA Aquagen – твій must-have для глибокого зволоження та сяючої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>520</t>
+  </si>
+  <si>
+    <t>Розкішний живильний крем з церамідами 50 мл</t>
+  </si>
+  <si>
+    <t>✨ Luxury Ceramide Nourishing Cream – глибоке живлення та сяйво! ✨
+🌿 Інноваційна формула для щоденного догляду:
+💧 Технологія подвійного зволоження – миттєвий та тривалий ефект
+🌸 Церамиди зміцнюють захисний бар’єр шкіри
+🥥 Комплекс Multifeel забезпечує інтенсивне живлення
+🌟 Пантенол заспокоює та відновлює
+💎 Зменшує глибину зморшок, підвищує пружність та еластичність
+💚 Результат – гладка, сяюча та здорова шкіра щодня!
+📌 Показання до застосування:
+Суха та зневоднена шкіра
+Зріла та чутлива шкіра
+Всі типи шкіри для щоденного догляду
+Відновлення після косметичних процедур
+✔️ Характеристики продукту:
+Тип: Живильний крем з церамідами
+Об’єм: 50 мл / 100 мл (залежно від упаковки)
+Призначення: Зволоження, живлення, відновлення, омолодження
+Тип шкіри: Всі типи, особливо суха та зріла
+Країна виробництва: 🇺🇦 Україна
+🌟 Luxury Ceramide Nourishing Cream – твій must-have для глибокого живлення та сяючої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>525</t>
+  </si>
+  <si>
+    <t>Невагомий Крем-гель SPF 50 - 50 мл</t>
+  </si>
+  <si>
+    <t>✨ Weightless SPF 50 Gel-Cream – щоденний захист та зволоження! ✨
+🌿 Інноваційна формула для комфортного щоденного догляду:
+☀️ Потужний УФ-захист: комплекс PolyFructol Plus та X50 Skin Barrier запобігає фотостарінню та передчасним зморшкам
+💧 Глибоке зволоження: технологія PatcH2O та Hydagen® Aquaporine працюють на клітинному рівні
+🛡️ Антиоксидантний захист: DN-Age нейтралізує вільні радикали та стрес
+🌸 Легка текстура: миттєво вбирається без липкості, даруючи комфорт
+💚 Результат – пружна, гладка та захищена шкіра з ефектом свіжості після кожного нанесення!
+📌 Показання до застосування:
+Щоденний догляд для всіх типів шкіри
+Захист від фото- та хроностаріння
+Профілактика зморшок та пігментації
+Зволоження та підтримка клітинного балансу
+📌 Як застосовувати:  
+Наносити на чисту, суху шкіру обличчя за 20 хвилин до виходу на сонце. Використовувати щодня для максимального захисту.
+✔️ Характеристики продукту:
+Тип: Крем-гель з SPF
+Об’єм: 50 мл / 230 мл
+Рівень захисту: SPF 50+ PA++++
+Призначення: Захист, зволоження, антиоксидантний догляд
+Тип шкіри: Всі типи
+Країна виробництва: 🇺🇦 Україна
+🌟 Weightless SPF 50 Gel-Cream – твій must-have для щоденного захисту та сяючої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>524</t>
+  </si>
+  <si>
+    <t>Постпроцедурний захисний регенерувальний спрей SPF50, 150 мл</t>
+  </si>
+  <si>
+    <t>518</t>
+  </si>
+  <si>
+    <t>✨ Post-Procedure Protective Spray SPF 50 – професійний догляд та відновлення! ✨
+🌿 Інноваційна формула для чутливої та пошкодженої шкіри:
+☀️ Максимальний захист SPF 50 від UVA/UVB-випромінювання
+💧 Відновлює оптимальний рівень зволоження без відчуття важкості
+🌸 Заспокоює подразнення та зменшує сухість
+🛡️ Сприяє регенерації та відновленню бар’єрної функції
+⚡ Зручний формат спрею для рівномірного нанесення
+💚 Результат – захищена, зволожена та відновлена шкіра після процедур!
+📌 Показання до застосування:
+Догляд після пілінгів, лазерних процедур, шліфування
+Суха та чутлива шкіра
+Роздратування та зневоднення
+Зниження тонусу та перші ознаки старіння
+Відновлення бар’єрної функції
+✔️ Характеристики продукту:
+Тип: Захисний регенерувальний спрей
+Об’єм: 150 мл
+Фактор захисту: SPF 50
+Спектр: UVA/UVB
+Водостійкий, гіпоалергенний
+Без вікових обмежень
+Країна виробництва: 🇺🇦 Україна
+🌟 Post-Procedure Protective Spray SPF 50 – твій must-have для безпечного та комфортного відновлення шкіри після процедур! 🌟</t>
+  </si>
+  <si>
+    <t>Сонцезахисний ультразволожувальний крем SPF50 з олією канабісу 50 мл</t>
+  </si>
+  <si>
+    <t>✨ Cannabis Ultra-Hydrating Sunscreen SPF 50 – повний спектр захисту та сяйво! ✨
+🌿 Інноваційна формула для щоденного догляду:
+☀️ SPF50 + широкоспектральний UVA/UVB-захист – профілактика фотостаріння та збереження колагену
+💧 Гіалуронова кислота + PolyFructol Plus – глибоке зволоження та підтримка водного балансу
+🌸 Екстракт азіатської центелли – заспокоює та відновлює бар’єрні функції
+🛡️ Токоферол ацетат та аскорбіл глюкозид – антиоксидантний захист від стресу та вільних радикалів
+🌟 Легка текстура з матуючим ефектом – без відчуття тяжкості
+💚 Результат – пружна, сяюча та захищена шкіра щодня!
+📌 Показання до застосування:
+Суха та чутлива шкіра
+Подразнення та зневоднення
+Перші ознаки старіння
+Зниження бар’єрної функції
+📌 Як застосовувати:  
+Наносити на очищену шкіру обличчя вранці, за 20 хвилин до виходу на сонце. Використовувати щодня для максимального ефекту.
+✔️ Характеристики продукту:
+Тип: Сонцезахисний крем з SPF
+Об’єм: 50 мл
+Рівень захисту: SPF 50+ PA++++
+Призначення: Захист, зволоження, антиоксидантний догляд
+Тип шкіри: Суха, чутлива, зріла
+Країна виробництва: 🇺🇦 Україна
+🌟 Cannabis Ultra-Hydrating Sunscreen SPF 50 – твій must-have для щоденного захисту та сяйва шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>517</t>
+  </si>
+  <si>
+    <t>Ультразволожуючий бустер х50 "Поліфруктол", 30 мл</t>
+  </si>
+  <si>
+    <t>510</t>
+  </si>
+  <si>
+    <t>✨ Polyfructol x50 Ultra-Hydrating Booster – інноваційна енергія зволоження! ✨
+🌿 Передова дрон-молекулярна система доставки:
+💧 Миттєва, глибока та пролонгована гідратація
+🌸 Стимулює природне продукування гіалуронової кислоти
+🛡️ Відновлює водний баланс та бар’єрні функції шкіри
+⚡ Зменшує запальні процеси та подразнення
+🌟 Покращує текстуру та еластичність
+💚 Результат – шкіра стає свіжою, пружною та сяючою вже після першого застосування!
+📌 Ключові активні компоненти:
+🌱 Skin Barrier та Polyfructol Plus – захист та пролонговане зволоження
+🌿 Олія коноплі та екстракт зеленого чаю – антиоксидантний щит та живлення
+💧 Бета-глюкан, трегалоза, альгін – глибоке зволоження та відновлення
+🌸 Purisoft™ LS 9836 – детокс та захист від зовнішніх факторів
+📌 Показання до застосування:
+Суха та чутлива шкіра
+Подразнення та зневоднення
+Зниження тонусу та перші ознаки старіння
+Відновлення бар’єрної функції
+✔️ Характеристики продукту:
+Тип: Антиоксидантний ультразволожуючий бустер
+Об’єм: 30 мл
+Призначення: Зволоження, живлення, антиоксидантний захист
+Тип шкіри: Суха, чутлива, зріла
+Країна виробництва: 🇺🇦 Україна
+🌟 Polyfructol x50 Booster – твій must-have для екстра зволоження та сяйва шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>Удосконалювало ний зволожувальний СС КРЕМ SPF30 - 50 мл</t>
+  </si>
+  <si>
+    <t>✨ Advanced Moisturizing CC Cream SPF 30 – ідеальний тон та захист! ✨
+🌿 Мультифункціональна формула для щоденного догляду:
+💎 Пігменти в мікрокапсулах адаптуються до відтінку шкіри
+🌸 Вирівнює тон та дарує миттєвий ефект свіжості
+☀️ Захист від ультрафіолету завдяки SPF 30
+💧 Легка текстура – не забиває пори та забезпечує комфорт
+💚 Результат – рівний тон, сяйво та захищена шкіра щодня!
+📌 Ключові активні компоненти:
+🥥 Масло насіння жожоба та ши – живлення та м’якість
+🌿 Екстракт камелії – стимуляція регенерації
+💧 Гіалуронат натрію – інтенсивне зволоження
+🛡️ Оксид цинку – захист від UVA/UVB-променів
+🌸 Пчелиний віск – заспокоює та утримує вологу
+⚡ Ацетил гексапептид-8 – зменшення зморшок
+🌟 Вітамін Е та лецитин – антиоксидантний захист та баланс
+📌 Як застосовувати:  
+Нанеси крем на чисту шкіру обличчя, шиї та декольте масажними рухами. Використовуй щодня для рівного тону та захисту від сонця.
+✔️ Характеристики продукту:
+Тип: Зволожувальний СС крем з SPF
+Об’єм: 50 мл
+Рівень захисту: SPF 30
+Призначення: Тонування, зволоження, захист, омолодження
+Тип шкіри: Всі типи, особливо суха та чутлива
+Країна виробництва: 🇺🇦 Україна
+🌟 Advanced CC Cream SPF 30 – твій must-have для ідеального тону та щоденного захисту! 🌟</t>
+  </si>
+  <si>
+    <t>519</t>
+  </si>
+  <si>
+    <t>Екстразволожувальний крем із церамідами SPF30 суха та нормальна шкіра</t>
+  </si>
+  <si>
+    <t>✨ Ceramide Extra-Hydrating Cream SPF 30 – подвійний захист та зволоження! ✨
+🌿 Інноваційна формула для щоденного догляду:
+💧 Комплекс церамідів I–IV, VI – відновлює бар’єрну функцію та зміцнює шкіру
+🌸 Гіалуронова кислота + гліцерил глюкозид – пролонговане зволоження на клітинному рівні
+🛡️ Антиоксидантний щит – ферулова кислота, токоферол ацетат та екстракт зеленого чаю нейтралізують вільні радикали
+☀️ SPF 30 широкого спектру – невидимий сонцезахисний щит проти UVA/UVB
+🌟 PatcH20 та Hydagen® Aquaporin – підтримка водного балансу та пружності
+💚 Результат – гладка, сяюча та захищена шкіра без сухості та подразнень!
+📌 Показання до застосування:
+Суха та чутлива шкіра
+Подразнення та зневоднення
+Зниження тонусу та перші ознаки старіння
+Відновлення та захист бар’єрної функції
+📌 Активні компоненти:
+🌱 Оливкова олія, екстракт ромашки, центелла азіатська
+💧 Hydagen® Aquaporin, PatcH20, Д-пантенол
+🛡️ iActive Ceramide, X50 Skin Barrier, Phytosoothe LS 9766
+🌸 Токоферол ацетат, натрій аскорбіл фосфат, ферулова кислота, бісаболол
+✔️ Характеристики продукту:
+Тип: Екстразволожувальний крем із SPF
+Об’єм: 50 мл
+Рівень захисту: SPF 30
+Призначення: Зволоження, живлення, антиоксидантний захист, сонцезахист
+Тип шкіри: Суха, нормальна, чутлива
+Країна виробництва: 🇺🇦 Україна
+🌟 Ceramide Extra-Hydrating Cream SPF 30 – твій must-have для щоденного зволоження та захисту шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>506</t>
+  </si>
+  <si>
+    <t>Крем-маска глибоке зволоження 50 мл</t>
+  </si>
+  <si>
+    <t>✨ Deep Moisture Cream-Mask – миттєве та пролонговане зволоження! ✨
+🌿 Легка пептидна формула з системою доставки X50:
+💧 Створює депо вологи в шкірі для подвійного ефекту гідратації
+🌸 Відновлює бар’єрні функції завдяки комплексу церамідів
+🛡️ Заспокоює подразнення та зменшує сухість
+⚡ Підвищує тонус та еластичність шкіри
+🌟 Дарує свіжість і сяйво вже після першого застосування
+💚 Результат – шкіра стає пружною, гладкою та сяючою!
+📌 Показання до застосування:
+Суха та чутлива шкіра
+Подразнення та зневоднення
+Зниження тонусу
+Перші ознаки старіння
+Відновлення та захист шкіри
+📌 Ключові активні компоненти:
+💧 Hydagen® Aquaporin, гіалуронат натрію, PolyFructol Plus – інтенсивне зволоження
+🌱 Олія авокадо, примули, екстракт центелли – живлення та відновлення
+🌸 Д-пантенол, ніацинамід, бета-глюкан – заспокійливий та регенеруючий ефект
+🛡️ iActive Ceramide, X50 Skin Barrier, токоферол, ферулова кислота, убіхінон – антиоксидантний захист та зміцнення бар’єру
+⚡ Амінокислоти та магнезіум аскорбіл фосфат – стимуляція клітинного оновлення
+✔️ Характеристики продукту:
+Тип: Крем-маска для глибокого зволоження
+Об’єм: 300 мл
+Призначення: Зволоження, живлення, відновлення, антиоксидантний захист
+Тип шкіри: Суха, чутлива, зріла
+Країна виробництва: 🇺🇦 Україна
+🌟 Deep Moisture Cream-Mask – твій must-have для миттєвого та тривалого зволоження! 🌟</t>
+  </si>
+  <si>
+    <t>514</t>
+  </si>
+  <si>
+    <t>Зволожувальний дренажний крем від темних кіл та набряків 30 мл</t>
+  </si>
+  <si>
+    <t>✨ Drainage Moisturizing Eye Cream – свіжий та сяючий погляд! ✨
+🌿 Активна формула для зони навколо очей:
+💧 Інтенсивне зволоження та відновлення бар’єрної функції
+🌸 Освітлення темних кіл завдяки екстракту водоростей
+🛡️ Зменшення набряків завдяки рутину та ескуліну
+⚡ Комплекс інкапсульованих пептидів – стимуляція синтезу білків для пружності
+🌟 Живлення та захист завдяки олії авокадо та примули
+💚 Результат – зменшені набряки, світліший тон та пружна шкіра навколо очей!
+📌 Активні компоненти:
+🌱 Екстракт водоростей – покращує кровообіг та освітлює темні кола
+🌸 Рутин + ескулін – протинабрякова дія
+💧 Інулін – підвищує пружність та еластичність
+⚡ Інкапсульовані пептиди – стимулюють синтез кератину, філагрину та лорекину
+🥥 Олія авокадо та примули вечірньої – живлення та захист
+🌟 Токоферол + магнезіум аскорбіл фосфат – антиоксидантний щит
+📌 Показання до застосування:
+Суха та чутлива шкіра навколо очей
+Подразнення та зневоднення
+Зниження тонусу
+Перші ознаки старіння
+Відновлення бар’єрної функції
+✔️ Характеристики продукту:
+Тип: Зволожувальний дренажний крем для очей
+Об’єм: 30 мл
+Призначення: Зволоження, протинабрякова дія, освітлення темних кіл
+Тип шкіри: Суха, чутлива, зріла
+Країна виробництва: 🇺🇦 Україна
+🌟 Drainage Moisturizing Eye Cream – твій must-have для сяючого та відпочилого погляду! 🌟</t>
+  </si>
+  <si>
+    <t>508</t>
+  </si>
+  <si>
+    <t>Дренажна освітлююча маска Глабрідин для очей 50 мл</t>
+  </si>
+  <si>
+    <t>✨ Smart4Derma Glabridin Eye Mask – професійний догляд для сяючого погляду! ✨
+🌿 Інноваційна формула для переорбітальної зони:
+💧 Зволожує та підвищує еластичність шкіри
+🌸 Освітлює темні кола та зменшує набряки нижніх повік
+🛡️ Зміцнює судини та покращує мікроциркуляцію
+⚡ Активізує виведення заліза та білірубіну, зменшуючи тьмяність
+🌟 Відновлює бар’єрну функцію та захищає від стресових факторів
+💚 Результат – свіжий, відпочилий та сяючий погляд!
+📌 Активні компоненти:
+🌱 Shadownyl, Рутин, Ескулін – зміцнення судин та протинабрякова дія
+🌸 Inoveol EGCG, екстракт зеленого чаю та каштана – антиоксидантний захист та покращення кровообігу
+💧 PolyFructol Plus, Hydagen® Aquaporin, інулін – глибоке зволоження та підтримка водного балансу
+🛡️ X50® Skin Barrier та комплекс пептидів – стимуляція синтезу кератину та філагрину, відновлення бар’єру
+📌 Показання до застосування:
+Суха та чутлива шкіра навколо очей
+Подразнення та зневоднення
+Зниження тонусу
+Перші ознаки старіння
+Відновлення та захист
+✔️ Характеристики продукту:
+Тип: Дренажна освітлююча маска для очей
+Об’єм: 50 мл
+Призначення: Зволоження, освітлення, протинабрякова дія, відновлення
+Бренд: Smart4Derma (Україна + Німеччина)
+Країна виробництва: 🇺🇦 Україна / 🇩🇪 Німеччина
+🌟 Smart4Derma Glabridin Eye Mask – твій must-have для сяючого та відпочилого погляду! 🌟</t>
+  </si>
+  <si>
+    <t>512</t>
+  </si>
+  <si>
+    <t>Екстразволожувальна Антиоксидантна сиворотка з центеллою 50 мл</t>
+  </si>
+  <si>
+    <t>✨ Smart4Derma Glabridin Eye Mask – професійний догляд для сяючого погляду! ✨
+🌿 Комплексне рішення для делікатної переорбітальної зони:
+💧 Інтенсивне зволоження та підвищення еластичності
+🌸 Освітлення темних кіл та зменшення набряків нижніх повік
+🛡️ Зміцнення судин та покращення мікроциркуляції
+⚡ Активізація процесів виведення заліза та білірубіну для рівного тону
+🌟 Відновлення бар’єрної функції та захист від стресових факторів
+💚 Результат – свіжий, відпочилий та сяючий погляд без ознак втоми!
+📌 Активні компоненти:
+🌱 Shadownyl, Рутин, Ескулін – протинабрякова дія та зміцнення судин
+🌸 Inoveol EGCG, екстракти зеленого чаю та каштана – антиоксидантний захист і покращення кровообігу
+💧 PolyFructol Plus, Hydagen® Aquaporin, інулін – глибоке та пролонговане зволоження
+🛡️ X50® Skin Barrier та комплекс пептидів – стимуляція синтезу кератину та філагрину, відновлення бар’єру
+📌 Показання до застосування:
+Суха та чутлива шкіра навколо очей
+Подразнення та зневоднення
+Зниження тонусу
+Перші ознаки старіння
+Відновлення та захист
+✔️ Характеристики продукту:
+Тип: Дренажна освітлююча маска для очей
+Об’єм: 50 мл
+Призначення: Зволоження, освітлення, протинабрякова дія, відновлення
+Бренд: Smart4Derma (🇺🇦 Україна + 🇩🇪 Німеччина)
+🌟 Smart4Derma Glabridin Eye Mask – твій must-have для сяючого та відпочилого погляду! 🌟</t>
+  </si>
+  <si>
+    <t>509</t>
+  </si>
+  <si>
+    <t>Зволожуючий гель-тонер для сіяння шкіри 250 мл</t>
+  </si>
+  <si>
+    <t>✨ Polyfructol Toner Bright Skin – професійне сяйво та зволоження! ✨
+🌿 Інноваційна формула для атонічної та зневодненої шкіри:
+💧 Hydagen® Aquaporin + PatcH2O – інтенсивне зволоження та утримання вологи
+🌸 Екстракти ромашки та шавлії – заспокоюють, знімають почервоніння та дискомфорт
+🌟 Ніацинамід – вирівнює тон та додає природне сяйво
+🛡️ Puricare POE LS 9727 + PolyFructol Plus – захист від негативного впливу навколишнього середовища
+⚡ Д-пантенол та натрій гіалуронат – пружність та відчуття свіжості
+💚 Результат – тривале зволоження до 24 годин, свіжий вигляд та сяюча шкіра!
+📌 Результати використання:
+Тривале зволоження на 24 години
+Свіжий та сяючий вигляд шкіри
+Активація процесів оновлення клітин та синтезу колагену
+Захист та покращення бар’єрної функції
+✔️ Характеристики продукту:
+Тип: Зволожуючий гель-тонер
+Об’єм: 250 мл
+Призначення: Зволоження, сяйво, захист
+Тип шкіри: Суха, тьмяна, атонічна
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Polyfructol Toner Bright Skin – твій must-have для сяючої та зволоженої шкіри щодня! 🌟</t>
+  </si>
+  <si>
+    <t>505</t>
+  </si>
+  <si>
+    <t>Пінка для сухої та чутливої шкіри з канабісом Hydro Aloe Mousse 80 мл</t>
+  </si>
+  <si>
+    <t>✨ Luxury Gentle Cleansing Foam – делікатне очищення та зволоження! ✨
+🌿 Спеціальна формула для щоденного догляду:
+💧 Легка текстура ефективно видаляє забруднення та макіяж
+🌸 Вирівнює поверхню шкіри без відчуття стягнутості
+🛡️ Заспокоює подразнення та зменшує запалення
+🌟 Відновлює бар’єрні функції та дарує відчуття комфорту
+💚 Результат – чиста, м’яка та сяюча шкіра після кожного очищення!
+📌 Активні компоненти:
+🌱 Олія коноплі та чіа – насичені омега-кислотами, зменшують подразнення
+🌸 Екстракт ромашки – заспокоює чутливу шкіру
+💧 Інулін та Hydagen® Aquaporin – глибоке зволоження та еластичність
+🛡️ Д-пантенол та бетаїн – відновлення та захист бар’єру
+📌 Показання до застосування:
+Суха та чутлива шкіра
+Подразнення та зневоднення
+Зниження тонусу
+Перші ознаки старіння
+Відновлення бар’єрної функції
+✔️ Характеристики продукту:
+Тип: Очищувальна піна для обличчя
+Об’єм: 150 мл / 200 мл (залежно від упаковки)
+Призначення: Делікатне очищення, зволоження, відновлення
+Тип шкіри: Суха, чутлива
+Країна виробництва: 🇺🇦 Україна
+🌟 Luxury Gentle Cleansing Foam – твій must-have для щоденного ніжного очищення та сяйва шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>504</t>
+  </si>
+  <si>
+    <t>Розкішне молочко для вмивання ОМЕГА Smart Derma 250 мл ніжне очищення</t>
+  </si>
+  <si>
+    <t>✨ Gentle Omega Cleansing – делікатне очищення та регенерація! ✨
+🌿 Багатофункціональна формула для щоденного догляду:
+💧 Ефективно видаляє макіяж та всі типи забруднень (водо- і жиророзчинні)
+🌸 Відновлює та інтенсивно регенерує шкіру
+🛡️ Попереджає подразнення та зневоднення
+⚡ Підтримує водно-ліпідний баланс
+🌟 Активізує кровообіг та покращує тургор
+💚 Результат – чиста, свіжа та сяюча шкіра без відчуття сухості!
+📌 Активні компоненти:
+🌱 Олія коноплі та чіа – насичені омега-кислотами, живлення та протизапальна дія
+🌸 Екстракт ромашки та центелли азіатської – заспокоюють та відновлюють
+💧 Hydagen® Aquaporin, PatcH2O, сечовина – інтенсивне зволоження та утримання вологи
+🛡️ Д-пантенол та натрій аскорбіл фосфат – антиоксидантний захист та регенерація
+📌 Показання до застосування:
+Суха та чутлива шкіра
+Подразнення та зневоднення
+Зниження тонусу
+Перші ознаки старіння
+Відновлення та захист бар’єрної функції
+✔️ Характеристики продукту:
+Тип: Очищуючий засіб для обличчя
+Об’єм: 150 мл / 200 мл (залежно від упаковки)
+Призначення: Очищення, регенерація, зволоження
+Тип шкіри: Суха, чутлива
+Країна виробництва: 🇺🇦 Україна
+🌟 Gentle Omega Cleansing – твій must-have для щоденного делікатного очищення та сяйва шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>500</t>
+  </si>
+  <si>
+    <t>Мультикислотна локальна присушка 50 мл</t>
+  </si>
+  <si>
+    <t>✨ LOCAL SOS Lotion – точковий удар по акне! ✨
+🌿 Високоефективна мультикислотна формула для проблемної шкіри:
+💧 Сірка та камфора – антибактеріальна та протизапальна дія
+🌸 Саліцилова кислота – глибоке очищення пор
+🛡️ Нікотинамід та оксид цинку – заспокоюють, відновлюють та створюють захисний бар’єр
+⚡ Азелаїнова, мигдальна та молочна кислоти – вирівнюють тон та борються з постакне
+🌟 Bix'Activ + екстракт каштана – зменшують почервоніння та регулюють себум
+💚 Результат – зменшення запалень, швидке підсушування висипань та відновлена шкіра!
+📌 Показання до застосування:
+Акне 1–3 ступеня
+Постакне та розширені пори
+Нерівний тон шкіри
+Атопічний дерматит, псоріаз, екзема
+Подразнення та свербіж
+📌 Додаткові активні компоненти:
+🌱 Д-пантенол – заспокоює та регенерує
+💧 Гліцерин – підтримує зволоження
+⚡ Кофеїн – активізує мікроциркуляцію
+✔️ Характеристики продукту:
+Тип: Локальний засіб для проблемної шкіри
+Об’єм: 50 мл
+Призначення: Підсушування, протизапальна дія, відновлення
+Тип шкіри: Проблемна, жирна, комбінована
+Лінія: Акнедерм
+Країна виробництва: 🇺🇦 Україна
+🌟 LOCAL SOS Lotion – твій must-have для швидкої допомоги при акне та подразненнях! 🌟</t>
+  </si>
+  <si>
+    <t>410</t>
   </si>
 </sst>
 </file>
@@ -5557,9 +6195,11 @@
         <v>658</v>
       </c>
       <c r="D5" s="8">
+        <v>1300</v>
+      </c>
+      <c r="E5" s="8">
         <v>1100</v>
       </c>
-      <c r="E5" s="8"/>
       <c r="F5" s="8"/>
       <c r="G5" s="8">
         <v>31</v>
@@ -5588,9 +6228,11 @@
         <v>658</v>
       </c>
       <c r="D6" s="8">
+        <v>1200</v>
+      </c>
+      <c r="E6" s="8">
         <v>1100</v>
       </c>
-      <c r="E6" s="8"/>
       <c r="F6" s="8"/>
       <c r="G6" s="8">
         <v>15</v>
@@ -7345,294 +7987,608 @@
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A63" s="12"/>
-      <c r="B63" s="8"/>
+      <c r="A63" s="12" t="s">
+        <v>843</v>
+      </c>
+      <c r="B63" s="8" t="s">
+        <v>841</v>
+      </c>
       <c r="C63" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D63" s="8"/>
+      <c r="D63" s="8">
+        <v>1140</v>
+      </c>
       <c r="E63" s="8"/>
       <c r="F63" s="8"/>
-      <c r="G63" s="8"/>
-      <c r="H63" s="8"/>
+      <c r="G63" s="8">
+        <v>16</v>
+      </c>
+      <c r="H63" s="8" t="s">
+        <v>43</v>
+      </c>
       <c r="I63" s="8" t="s">
         <v>657</v>
       </c>
-      <c r="J63" s="8"/>
-      <c r="K63" s="18"/>
+      <c r="J63" s="8" t="s">
+        <v>842</v>
+      </c>
+      <c r="K63" s="18" t="s">
+        <v>843</v>
+      </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A64" s="12"/>
-      <c r="B64" s="8"/>
+      <c r="A64" s="12" t="s">
+        <v>846</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>844</v>
+      </c>
       <c r="C64" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D64" s="8"/>
+      <c r="D64" s="8">
+        <v>1000</v>
+      </c>
       <c r="E64" s="8"/>
       <c r="F64" s="8"/>
-      <c r="G64" s="8"/>
-      <c r="H64" s="8"/>
+      <c r="G64" s="8">
+        <v>19</v>
+      </c>
+      <c r="H64" s="8" t="s">
+        <v>672</v>
+      </c>
       <c r="I64" s="8" t="s">
         <v>657</v>
       </c>
-      <c r="J64" s="8"/>
-      <c r="K64" s="18"/>
+      <c r="J64" s="8" t="s">
+        <v>845</v>
+      </c>
+      <c r="K64" s="18" t="s">
+        <v>846</v>
+      </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A65" s="12"/>
-      <c r="B65" s="8"/>
+      <c r="A65" s="12" t="s">
+        <v>849</v>
+      </c>
+      <c r="B65" s="8" t="s">
+        <v>847</v>
+      </c>
       <c r="C65" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D65" s="8"/>
+      <c r="D65" s="8">
+        <v>780</v>
+      </c>
       <c r="E65" s="8"/>
       <c r="F65" s="8"/>
-      <c r="G65" s="8"/>
-      <c r="H65" s="8"/>
+      <c r="G65" s="8">
+        <v>16</v>
+      </c>
+      <c r="H65" s="8" t="s">
+        <v>672</v>
+      </c>
       <c r="I65" s="8" t="s">
         <v>657</v>
       </c>
-      <c r="J65" s="8"/>
-      <c r="K65" s="18"/>
+      <c r="J65" s="8" t="s">
+        <v>848</v>
+      </c>
+      <c r="K65" s="18" t="s">
+        <v>849</v>
+      </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A66" s="12"/>
-      <c r="B66" s="8"/>
+      <c r="A66" s="12" t="s">
+        <v>853</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>850</v>
+      </c>
       <c r="C66" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D66" s="8"/>
+      <c r="D66" s="8">
+        <v>1320</v>
+      </c>
       <c r="E66" s="8"/>
       <c r="F66" s="8"/>
-      <c r="G66" s="8"/>
-      <c r="H66" s="8"/>
+      <c r="G66" s="8">
+        <v>19</v>
+      </c>
+      <c r="H66" s="8" t="s">
+        <v>851</v>
+      </c>
       <c r="I66" s="8" t="s">
         <v>657</v>
       </c>
-      <c r="J66" s="8"/>
-      <c r="K66" s="18"/>
+      <c r="J66" s="8" t="s">
+        <v>852</v>
+      </c>
+      <c r="K66" s="18" t="s">
+        <v>853</v>
+      </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A67" s="12"/>
-      <c r="B67" s="8"/>
+      <c r="A67" s="12" t="s">
+        <v>856</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>854</v>
+      </c>
       <c r="C67" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D67" s="8"/>
+      <c r="D67" s="8">
+        <v>680</v>
+      </c>
       <c r="E67" s="8"/>
       <c r="F67" s="8"/>
-      <c r="G67" s="8"/>
-      <c r="H67" s="8"/>
+      <c r="G67" s="8">
+        <v>25</v>
+      </c>
+      <c r="H67" s="8" t="s">
+        <v>43</v>
+      </c>
       <c r="I67" s="8" t="s">
         <v>657</v>
       </c>
-      <c r="J67" s="8"/>
-      <c r="K67" s="18"/>
+      <c r="J67" s="8" t="s">
+        <v>855</v>
+      </c>
+      <c r="K67" s="18" t="s">
+        <v>856</v>
+      </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A68" s="12"/>
-      <c r="B68" s="8"/>
+      <c r="A68" s="12" t="s">
+        <v>859</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>857</v>
+      </c>
       <c r="C68" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D68" s="8"/>
+      <c r="D68" s="8">
+        <v>980</v>
+      </c>
       <c r="E68" s="8"/>
       <c r="F68" s="8"/>
-      <c r="G68" s="8"/>
-      <c r="H68" s="8"/>
+      <c r="G68" s="8">
+        <v>17</v>
+      </c>
+      <c r="H68" s="8" t="s">
+        <v>43</v>
+      </c>
       <c r="I68" s="8" t="s">
         <v>657</v>
       </c>
-      <c r="J68" s="8"/>
-      <c r="K68" s="18"/>
+      <c r="J68" s="8" t="s">
+        <v>858</v>
+      </c>
+      <c r="K68" s="18" t="s">
+        <v>859</v>
+      </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A69" s="12"/>
-      <c r="B69" s="8"/>
+      <c r="A69" s="12" t="s">
+        <v>861</v>
+      </c>
+      <c r="B69" s="8" t="s">
+        <v>860</v>
+      </c>
       <c r="C69" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D69" s="8"/>
+      <c r="D69" s="8">
+        <v>1260</v>
+      </c>
       <c r="E69" s="8"/>
       <c r="F69" s="8"/>
-      <c r="G69" s="8"/>
-      <c r="H69" s="8"/>
+      <c r="G69" s="8">
+        <v>21</v>
+      </c>
+      <c r="H69" s="8" t="s">
+        <v>695</v>
+      </c>
       <c r="I69" s="8" t="s">
         <v>657</v>
       </c>
-      <c r="J69" s="8"/>
-      <c r="K69" s="18"/>
+      <c r="J69" s="8" t="s">
+        <v>862</v>
+      </c>
+      <c r="K69" s="18" t="s">
+        <v>861</v>
+      </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A70" s="12"/>
-      <c r="B70" s="8"/>
+      <c r="A70" s="12" t="s">
+        <v>865</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>863</v>
+      </c>
       <c r="C70" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D70" s="8"/>
+      <c r="D70" s="8">
+        <v>1020</v>
+      </c>
       <c r="E70" s="8"/>
       <c r="F70" s="8"/>
-      <c r="G70" s="8"/>
-      <c r="H70" s="8"/>
-      <c r="I70" s="8"/>
-      <c r="J70" s="8"/>
-      <c r="K70" s="18"/>
+      <c r="G70" s="8">
+        <v>26</v>
+      </c>
+      <c r="H70" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I70" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J70" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="K70" s="18" t="s">
+        <v>865</v>
+      </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A71" s="12"/>
-      <c r="B71" s="9"/>
-      <c r="C71" s="9"/>
-      <c r="D71" s="8"/>
+      <c r="A71" s="12" t="s">
+        <v>867</v>
+      </c>
+      <c r="B71" s="8" t="s">
+        <v>866</v>
+      </c>
+      <c r="C71" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D71" s="8">
+        <v>980</v>
+      </c>
       <c r="E71" s="8"/>
       <c r="F71" s="8"/>
-      <c r="G71" s="8"/>
-      <c r="H71" s="8"/>
-      <c r="I71" s="8"/>
-      <c r="J71" s="9"/>
-      <c r="K71" s="15"/>
+      <c r="G71" s="8">
+        <v>16</v>
+      </c>
+      <c r="H71" s="8" t="s">
+        <v>664</v>
+      </c>
+      <c r="I71" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J71" s="8" t="s">
+        <v>868</v>
+      </c>
+      <c r="K71" s="18" t="s">
+        <v>867</v>
+      </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A72" s="12"/>
-      <c r="B72" s="9"/>
-      <c r="C72" s="9"/>
-      <c r="D72" s="8"/>
+      <c r="A72" s="12" t="s">
+        <v>871</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>869</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D72" s="8">
+        <v>1220</v>
+      </c>
       <c r="E72" s="8"/>
       <c r="F72" s="8"/>
-      <c r="G72" s="8"/>
-      <c r="H72" s="8"/>
-      <c r="I72" s="8"/>
-      <c r="J72" s="9"/>
-      <c r="K72" s="15"/>
+      <c r="G72" s="8">
+        <v>17</v>
+      </c>
+      <c r="H72" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I72" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J72" s="8" t="s">
+        <v>870</v>
+      </c>
+      <c r="K72" s="18" t="s">
+        <v>871</v>
+      </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A73" s="12"/>
-      <c r="B73" s="9"/>
-      <c r="C73" s="9"/>
-      <c r="D73" s="8"/>
+      <c r="A73" s="12" t="s">
+        <v>874</v>
+      </c>
+      <c r="B73" s="8" t="s">
+        <v>872</v>
+      </c>
+      <c r="C73" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D73" s="8">
+        <v>1140</v>
+      </c>
       <c r="E73" s="8"/>
       <c r="F73" s="8"/>
-      <c r="G73" s="8"/>
-      <c r="H73" s="8"/>
-      <c r="I73" s="8"/>
-      <c r="J73" s="9"/>
-      <c r="K73" s="15"/>
+      <c r="G73" s="8">
+        <v>21</v>
+      </c>
+      <c r="H73" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I73" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J73" s="8" t="s">
+        <v>873</v>
+      </c>
+      <c r="K73" s="18" t="s">
+        <v>874</v>
+      </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A74" s="12"/>
-      <c r="B74" s="9"/>
-      <c r="C74" s="9"/>
-      <c r="D74" s="8"/>
+      <c r="A74" s="12" t="s">
+        <v>877</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>875</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D74" s="8">
+        <v>780</v>
+      </c>
       <c r="E74" s="8"/>
       <c r="F74" s="8"/>
-      <c r="G74" s="8"/>
-      <c r="H74" s="8"/>
-      <c r="I74" s="8"/>
-      <c r="J74" s="9"/>
-      <c r="K74" s="15"/>
+      <c r="G74" s="8">
+        <v>24</v>
+      </c>
+      <c r="H74" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I74" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J74" s="8" t="s">
+        <v>876</v>
+      </c>
+      <c r="K74" s="18" t="s">
+        <v>877</v>
+      </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A75" s="12"/>
-      <c r="B75" s="9"/>
-      <c r="C75" s="9"/>
-      <c r="D75" s="8"/>
+      <c r="A75" s="12" t="s">
+        <v>880</v>
+      </c>
+      <c r="B75" s="8" t="s">
+        <v>878</v>
+      </c>
+      <c r="C75" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D75" s="8">
+        <v>660</v>
+      </c>
       <c r="E75" s="8"/>
       <c r="F75" s="8"/>
-      <c r="G75" s="8"/>
-      <c r="H75" s="8"/>
-      <c r="I75" s="8"/>
-      <c r="J75" s="9"/>
-      <c r="K75" s="15"/>
+      <c r="G75" s="8">
+        <v>13</v>
+      </c>
+      <c r="H75" s="8" t="s">
+        <v>664</v>
+      </c>
+      <c r="I75" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J75" s="8" t="s">
+        <v>879</v>
+      </c>
+      <c r="K75" s="18" t="s">
+        <v>880</v>
+      </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A76" s="12"/>
-      <c r="B76" s="9"/>
-      <c r="C76" s="9"/>
-      <c r="D76" s="8"/>
+      <c r="A76" s="12" t="s">
+        <v>883</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>881</v>
+      </c>
+      <c r="C76" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D76" s="8">
+        <v>1000</v>
+      </c>
       <c r="E76" s="8"/>
       <c r="F76" s="8"/>
-      <c r="G76" s="8"/>
-      <c r="H76" s="8"/>
-      <c r="I76" s="8"/>
-      <c r="J76" s="9"/>
-      <c r="K76" s="15"/>
+      <c r="G76" s="8">
+        <v>14</v>
+      </c>
+      <c r="H76" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I76" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J76" s="8" t="s">
+        <v>882</v>
+      </c>
+      <c r="K76" s="18" t="s">
+        <v>883</v>
+      </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A77" s="12"/>
-      <c r="B77" s="9"/>
-      <c r="C77" s="9"/>
-      <c r="D77" s="8"/>
+      <c r="A77" s="12" t="s">
+        <v>886</v>
+      </c>
+      <c r="B77" s="8" t="s">
+        <v>884</v>
+      </c>
+      <c r="C77" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D77" s="8">
+        <v>1280</v>
+      </c>
       <c r="E77" s="8"/>
       <c r="F77" s="8"/>
-      <c r="G77" s="8"/>
-      <c r="H77" s="8"/>
-      <c r="I77" s="8"/>
-      <c r="J77" s="9"/>
-      <c r="K77" s="15"/>
+      <c r="G77" s="8">
+        <v>19</v>
+      </c>
+      <c r="H77" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I77" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J77" s="8" t="s">
+        <v>885</v>
+      </c>
+      <c r="K77" s="18" t="s">
+        <v>886</v>
+      </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A78" s="12"/>
-      <c r="B78" s="9"/>
-      <c r="C78" s="9"/>
-      <c r="D78" s="8"/>
+      <c r="A78" s="12" t="s">
+        <v>889</v>
+      </c>
+      <c r="B78" s="8" t="s">
+        <v>887</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D78" s="8">
+        <v>940</v>
+      </c>
       <c r="E78" s="8"/>
       <c r="F78" s="8"/>
-      <c r="G78" s="8"/>
-      <c r="H78" s="8"/>
-      <c r="I78" s="8"/>
-      <c r="J78" s="9"/>
-      <c r="K78" s="15"/>
+      <c r="G78" s="8">
+        <v>26</v>
+      </c>
+      <c r="H78" s="8" t="s">
+        <v>672</v>
+      </c>
+      <c r="I78" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J78" s="8" t="s">
+        <v>888</v>
+      </c>
+      <c r="K78" s="18" t="s">
+        <v>889</v>
+      </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A79" s="12"/>
-      <c r="B79" s="9"/>
-      <c r="C79" s="9"/>
-      <c r="D79" s="8"/>
+      <c r="A79" s="12" t="s">
+        <v>892</v>
+      </c>
+      <c r="B79" s="8" t="s">
+        <v>890</v>
+      </c>
+      <c r="C79" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D79" s="8">
+        <v>480</v>
+      </c>
       <c r="E79" s="8"/>
       <c r="F79" s="8"/>
-      <c r="G79" s="8"/>
-      <c r="H79" s="8"/>
-      <c r="I79" s="8"/>
-      <c r="J79" s="9"/>
-      <c r="K79" s="15"/>
+      <c r="G79" s="8">
+        <v>15</v>
+      </c>
+      <c r="H79" s="8" t="s">
+        <v>783</v>
+      </c>
+      <c r="I79" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J79" s="8" t="s">
+        <v>891</v>
+      </c>
+      <c r="K79" s="18" t="s">
+        <v>892</v>
+      </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A80" s="12"/>
-      <c r="B80" s="9"/>
-      <c r="C80" s="9"/>
-      <c r="D80" s="8"/>
+      <c r="A80" s="12" t="s">
+        <v>895</v>
+      </c>
+      <c r="B80" s="8" t="s">
+        <v>893</v>
+      </c>
+      <c r="C80" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D80" s="8">
+        <v>700</v>
+      </c>
       <c r="E80" s="8"/>
       <c r="F80" s="8"/>
-      <c r="G80" s="8"/>
-      <c r="H80" s="8"/>
-      <c r="I80" s="8"/>
-      <c r="J80" s="9"/>
-      <c r="K80" s="15"/>
+      <c r="G80" s="8">
+        <v>12</v>
+      </c>
+      <c r="H80" s="8" t="s">
+        <v>672</v>
+      </c>
+      <c r="I80" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J80" s="8" t="s">
+        <v>894</v>
+      </c>
+      <c r="K80" s="18" t="s">
+        <v>895</v>
+      </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A81" s="12"/>
-      <c r="B81" s="9"/>
-      <c r="C81" s="9"/>
-      <c r="D81" s="8"/>
+      <c r="A81" s="12" t="s">
+        <v>898</v>
+      </c>
+      <c r="B81" s="8" t="s">
+        <v>896</v>
+      </c>
+      <c r="C81" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D81" s="8">
+        <v>620</v>
+      </c>
       <c r="E81" s="8"/>
       <c r="F81" s="8"/>
-      <c r="G81" s="8"/>
-      <c r="H81" s="8"/>
-      <c r="I81" s="8"/>
-      <c r="J81" s="9"/>
-      <c r="K81" s="15"/>
+      <c r="G81" s="8">
+        <v>24</v>
+      </c>
+      <c r="H81" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I81" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J81" s="8" t="s">
+        <v>897</v>
+      </c>
+      <c r="K81" s="18" t="s">
+        <v>898</v>
+      </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A82" s="12"/>
-      <c r="B82" s="9"/>
-      <c r="C82" s="9"/>
+      <c r="B82" s="8"/>
+      <c r="C82" s="8"/>
       <c r="D82" s="8"/>
       <c r="E82" s="8"/>
       <c r="F82" s="8"/>
       <c r="G82" s="8"/>
       <c r="H82" s="8"/>
-      <c r="I82" s="8"/>
-      <c r="J82" s="9"/>
-      <c r="K82" s="15"/>
+      <c r="I82" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J82" s="8"/>
+      <c r="K82" s="18"/>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A83" s="12"/>

</xml_diff>

<commit_message>
feat: gift sets, smarter chat retrieval, Instagram contacts
- backend: optional Excel sheet sets builds gift sets (is_set/set_items,
  category Набори, auto price/stock/image, id set-*); UI badges +
  Склад набору block on product page
- chat: dynamic brand list in prompt, 10 hard rules, expandQuery synonyms,
  budget/sale boosts in retrieve, ensureThree, Instagram line in every reply
- footer/chat: @ua_cosmetics_lab links; docs: sets + new prompt verbatim
</commit_message>
<xml_diff>
--- a/data/price.xlsx
+++ b/data/price.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ПРОЕКТ AI\ЛИЧНЫЕ НАРАБОТКИ\AI Skin Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6108CA2E-69E2-4FCE-B252-B83B6657E986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D81DF18C-E7BA-43B2-91A7-A259D739512E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-1512" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Зручна таблиця" sheetId="1" r:id="rId1"/>
+    <sheet name="sets" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Зручна таблиця'!$A$1:$K$93</definedName>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1135" uniqueCount="569">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1374" uniqueCount="618">
   <si>
     <t>Артикул</t>
   </si>
@@ -5982,6 +5983,488 @@
   </si>
   <si>
     <t>AL302</t>
+  </si>
+  <si>
+    <t>Очищуюче молочко з екстрактом примули Anna Logor Vital Primrose Cleanser (Art.501), 350 мл</t>
+  </si>
+  <si>
+    <t>✨ Anna Logor Vital Primrose Cleanser – ніжне очищення та догляд після 30! ✨
+🌿 Чому варто обрати це молочко:
+💧 Делікатно видаляє макіяж та забруднення, не порушуючи баланс шкіри
+🌸 Живить та заспокоює, дарує відчуття комфорту
+🛡️ Сприяє регенерації клітин та захищає від шкідливих бактерій
+⚡ Допомагає боротися з першими ознаками старіння
+🌟 Підтримує пружність та свіжість шкіри
+💚 Результат – доглянута, сяюча та м’яка шкіра щодня!
+📌 Активні компоненти:
+🌱 Вітаміни А та С – антиоксидантний захист та омолодження
+🍋 Лимонна кислота – м’яке відлущування та вирівнювання тону
+🌸 Екстракти розмарину, хвої, примули, хвоща та хмелю – живлення, тонізація та регенерація
+📌 Основні властивості:
+Баланс вологи та живлення
+Заспокійлива дія та стимуляція регенерації
+Приємний аромат
+Легке нанесення та змивання теплою водою
+Економне використання завдяки дозатору
+📌 Спосіб застосування:
+Нанести молочко на ватний диск.
+Протерти шкіру від центру до країв, уникаючи зони навколо очей.
+Змити теплою водою.
+Для максимального ефекту використати тонік Vital Primrose.
+✔️ Характеристики продукту:
+Тип: Очищуюче молочко
+Об’єм: 350 мл
+Вікова категорія: 30+, без обмежень
+Призначення: Очищення, живлення, регенерація
+Бренд: Anna Logor
+Країна виробництва: 🇺🇦 Україна
+🌟 Anna Logor Vital Primrose Cleanser – твій must-have для ніжного догляду та збереження молодості шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>AL501</t>
+  </si>
+  <si>
+    <t>Тональний сонцезахисний крем SPF-30 UVA,UVB Anna Logor (Art.1057), 115 мл</t>
+  </si>
+  <si>
+    <t>115 мл</t>
+  </si>
+  <si>
+    <t>✨ Anna Logor Sunscreen SPF-30 – ідеальний тон та надійний захист! ✨
+🌿 Чому варто обрати цей крем:
+💧 Забезпечує рівний тон шкіри та тривале зволоження
+🌸 Захищає від UVA та UVB-променів, запобігаючи пігментації та зморшкам
+🛡️ Органічні, неорганічні та рослинні УФ-фільтри – ефективний захист від опіків і фотостаріння
+⚡ Сприяє регенерації клітин після пілінгу
+🌟 Гіпоалергенна формула, підходить навіть для жирної та комбінованої шкіри
+💚 Результат – свіжа, сяюча та захищена шкіра щодня!
+📌 Активні компоненти:
+🌱 Вітамін Е – антиоксидантний щит
+🌸 Екстракти мальви, бузини, огірка, плюща, настінниці лікарської, арніки – заспокоюють та відновлюють
+💧 Натуральні інгредієнти з вираженою регенеративною дією
+📌 Спосіб застосування:
+Очистіть шкіру обличчя та шиї за допомогою спеціального очищувача Anna Logor.
+Нанесіть крем рівномірним шаром перед виходом на сонце.
+Для тривалого ефекту повторюйте нанесення протягом дня.
+✔️ Характеристики продукту:
+Тип: Тональний сонцезахисний крем
+SPF: 30 (UVA/UVB)
+Об’єм: 115 мл · Туба з фліп-дозатором
+Призначення: Захист від сонця, вирівнювання тону, профілактика фотостаріння
+Тип шкіри: Усі типи, включно з жирною та комбінованою
+Бренд: Anna Logor
+Країна виробництва: 🇺🇦 Україна
+🌟 Anna Logor Sunscreen SPF-30 – твій must-have для рівного тону та бездоганного захисту від сонця! 🌟</t>
+  </si>
+  <si>
+    <t>AL1057</t>
+  </si>
+  <si>
+    <t>Тонік з екстрактом примули Anna Logor Vital Primrose Toner (Art.502), 350 мл</t>
+  </si>
+  <si>
+    <t>✨ Anna Logor Vital Primrose Toner – ніжний догляд та відновлення після 30! ✨
+🌿 Чому варто обрати цей тонік:
+💧 Делікатно видаляє забруднення та надлишки себуму
+🌸 Відновлює природний баланс вологи та рН
+🛡️ Заспокоює, пом’якшує та живить шкіру
+⚡ Сприяє швидкій регенерації клітин
+🌟 Допомагає боротися з першими ознаками старіння
+💚 Результат – доглянута, пружна та сяюча шкіра щодня!
+📌 Активні компоненти:
+🌱 Вітамін В5 – живлення та регенерація
+🌸 Екстракти розмарину, польового хвоща, примули, хмелю, лимона та хвої – тонізація, антиоксидантний захист та відновлення
+📌 Спосіб застосування:
+Використовуйте щодня вранці та ввечері після очищення обличчя молочком Anna Logor Vital Primrose Cleanser.
+Нанесіть тонік на ватний диск і акуратно протирайте шкіру по масажних лініях від центру до країв, уникаючи зони навколо очей.
+Для максимального ефекту після процедури застосуйте Mezotherapy Serum, Mezotherapy Firming Moisturizer або Mezotherapy Night Cream.
+✔️ Переваги продукту:
+Без спирту, делікатна формула
+Натуральні екстракти
+Підходить для щоденного використання
+Зручний флакон з дозатором
+🌟 Anna Logor Vital Primrose Toner – твій must-have для щоденного догляду та збереження молодості шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>AL502</t>
+  </si>
+  <si>
+    <t>Сонцезахисний крем SPF-50 UVA,UVB DD Cream Anna Logor (Art.1058), 110 мл</t>
+  </si>
+  <si>
+    <t>110 мл</t>
+  </si>
+  <si>
+    <t>✨ Anna Logor Sunscreen SPF-50 – максимальний захист та догляд! ✨
+🌿 Чому варто обрати цей крем:
+🛡️ Забезпечує надійний захист від UVA та UVB-променів
+💧 Запобігає фотостарінню та появі пігментації
+🌸 Інтенсивно зволожує та пом’якшує шкіру
+⚡ Сприяє відновленню клітин після впливу сонця чи косметологічних процедур
+🌟 Підходить для щоденного використання навіть на чутливій шкірі
+💚 Результат – свіжа, доглянута та захищена шкіра без відчуття жирності!
+📌 Активні компоненти:
+🌱 Аллантоїн – заспокоює та відновлює
+💧 Зволожуючий комплекс – підтримує баланс вологи
+🌸 Вітамін Е – антиоксидантний захист
+🌿 Екстракти мальви, плюща, постінниці лікарської, огірка, алое вера, бузини та арніки – живлення, тонізація та регенерація
+📌 Спосіб застосування:
+Очистіть шкіру обличчя та шиї за допомогою молочка чи пінного очищувача Anna Logor.
+Нанесіть невелику кількість крему круговими масажними рухами.
+Легкими дотиками пальців розподіліть до повного вбирання.
+✔️ Переваги продукту:
+Високий рівень захисту SPF-50
+Формула без подразнюючих компонентів
+Підходить для всіх типів шкіри, включно з чутливою
+Зручний флакон із дозатором для економного використання
+📦 Форма випуску:  
+Флакон із дозатором · 120 мл
+Формула: США · Виробництво: 🇺🇦 Україна
+🌟 Anna Logor Sunscreen SPF-50 – твій must-have для бездоганного захисту та здорової шкіри під сонцем! 🌟</t>
+  </si>
+  <si>
+    <t>AL1058</t>
+  </si>
+  <si>
+    <t>Очищуючий гель для жирної шкіри Anna Logor Oil Control Cleanser (Art.201), 350 мл</t>
+  </si>
+  <si>
+    <t>✨ Anna Logor Oil Control Cleanser – професійне очищення для жирної шкіри! ✨
+🌿 Чому варто обрати цей гель:
+💧 Регулює роботу сальних залоз
+🌸 Зменшує жирність та дарує матовість
+🛡️ Нормалізує рівень pH
+⚡ Ефективно видаляє забруднення, ороговілі клітини та залишки макіяжу
+🌟 Готує шкіру до наступних етапів догляду
+💚 Результат – чиста, свіжа та доглянута шкіра без жирного блиску!
+📌 Активні компоненти:
+🌱 Карбонова, себацинова та гідроксидексанова кислоти – м’яке відлущування, антибактеріальна дія, покращення мікрофлори
+🌸 Екстракти кори білої верби, лимона, лопуха, крес-салату, шавлії та плюща – природне очищення, тонізація та регенерація
+📌 Спосіб застосування:
+Нанесіть гель на вологу шкіру обличчя.
+Легко помасажуйте.
+Ретельно змийте теплою водою.
+Для максимального ефекту використовуйте стабілізуючий тонік Oil Control Toner Anna Logor.
+✔️ Переваги продукту:
+Легка текстура та приємний аромат
+Підходить для щоденного застосування
+Натуральний склад
+Зручний флакон із дозатором · 350 мл
+🌟 Anna Logor Oil Control Cleanser – твій must-have для щоденного догляду за жирною шкірою! 🌟</t>
+  </si>
+  <si>
+    <t>AL201</t>
+  </si>
+  <si>
+    <t>Інтенсивний ліфтинг-відновлюючий денний крем Perfect Skin Ultimate Lifting Recovery (Art.43), 50 мл</t>
+  </si>
+  <si>
+    <t>Інтенсивний ліфтинг-крем для глибокого відновлення
+Цей крем — потужний коктейль активних компонентів, що забезпечує глибоке відновлення та видимий ліфтинг. Формула працює одразу в трьох напрямках: екстремальне зволоження, зміцнення структури шкіри та захист від передчасного старіння.
+Основна дія
+✨ Миттєвий ліфтинг і гладкість Поєднання пуллулану, альгіну та інноваційного пептиду Palmitoyl Tripeptide-28 (з частинками сапфіру для кращого проникнення) підтягує овал обличчя та стимулює синтез колагену.
+💧 Глибоке 4D-зволоження Комплекс із гіалуронової кислоти, сечовини, трегалози та серину створює невидиму «дихаючу» сітку, яка утримує вологу протягом усього дня.
+🌿 Вітамінне омолодження Вітамін А прискорює оновлення клітин, а вітамін Е та глутатіон — один із найсильніших антиоксидантів — нейтралізують дію вільних радикалів і повертають шкірі сяйво.
+🌸 Живлення цінними оліями Олії примули вечірньої відновлюють захисний бар’єр, усувають сухість і дарують шкірі оксамитовість.
+🍃 Рослинний детокс Екстракти арніки, плюща та бузини знімають набряки, зміцнюють судини та вирівнюють тон обличчя.
+Кому підійде
+Ідеальний для зрілої, сухої або втомленої шкіри, що втратила тонус. Легка текстура на основі сквалану та сучасних емолентів швидко вбирається, не залишаючи жирного блиску, і чудово підходить як база під макіяж.
+Результат
+Шкіра стає більш щільною та підтягнутою
+Дрібні зморшки розгладжуються
+Обличчя виглядає свіжим, живленим і сяючим
+Застосування
+Наносити щодня вранці на очищене обличчя, шию та зону декольте. Для максимального ефекту рекомендується комбінувати з Visage Cream Rich 44 як нічним доглядом та використовувати разом із сироваткою.
+Активні компоненти
+Трипептид-28, зволожуючий комплекс PatchH2O™, сквалан, олії примули, пікуї, каштану, малини та крамбе, вітаміни А й Е, екстракти мальви, плюща, постенніци лікарської, огірка, бузини та арніки.
+Відчуття на шкірі
+Освіжає, ніжно зволожує, дарує шовковистість.
+Текстура
+Ніжна, повітряна, легка, швидко вбирається.
+Аромат
+Делікатна зелено-квіткова композиція з легким фруктовим відтінком.</t>
+  </si>
+  <si>
+    <t>AL43</t>
+  </si>
+  <si>
+    <t>Цитрусова маска для жирної шкіри Anna Logor Oil Control Citrus Mask (Art.255), 250 мл</t>
+  </si>
+  <si>
+    <t>✨ Anna Logor Oil Control Citrus Mask – свіжість та матовість для жирної шкіри! ✨
+🌿 Чому варто спробувати:
+💧 Регулює вироблення себуму
+🌸 Звужує пори та зменшує їх помітність
+🛡️ Знімає почервоніння та заспокоює шкіру
+⚡ Дарує матовий ефект і здоровий вигляд
+💚 Результат – чиста, доглянута та матова шкіра вже після першого застосування!
+📌 Активні компоненти:
+🌱 Себацинова та гідрокідеканова кислота – контроль себуму та м’яке відлущування
+🌸 Каолінова глина – очищення та матування
+🛡️ Органічна сірка – протизапальна дія
+🌿 Екстракти кресса водяного, лимона, гриба агарика, лопуха, плюща, шавлії – природне відновлення та захист
+🌟 Вітаміни А, Е, С – антиоксидантний комплекс
+📌 Консистенція та застосування:
+Ніжна пастоподібна текстура, легко наноситься та змивається
+Використовувати 1–2 рази на тиждень
+Нанести тонким шаром (1–2 мм) на очищену шкіру обличчя та шиї
+Через 15 хвилин змити прохолодною водою або видалити вологим рушником
+Для закріплення результату застосувати Oil Control Fluid Anna Logor
+✔️ Переваги продукту:
+Натуральний склад
+Швидкий ефект матування
+Приємний аромат
+Зручна форма випуску – баночка 250 мл · Art.255
+Вікова категорія: 16+
+🌟 Anna Logor Oil Control Citrus Mask – твій must-have для догляду за жирною шкірою та контролю себуму! 🌟</t>
+  </si>
+  <si>
+    <t>AL255</t>
+  </si>
+  <si>
+    <t>Живильний зміцнюючий нічний крем Perfect Skin Visage Cream Rich (Art.44), 50 мл</t>
+  </si>
+  <si>
+    <t>Нічний крем — «інтелектуальний відновлювач»
+Поки ви спите, крем працює над зміцненням каркаса шкіри, глибоким живленням та оновленням клітин. Вранці обличчя виглядає сяючим, свіжим і відпочилим.
+Основна дія
+✨ Пептидне моделювання (Drone Technology) Капсульована система доставки пептидів проникає у глибокі шари дерми, відновлює пошкоджені колагенові волокна, ущільнює шкіру та зменшує глибину зморшок.
+🌙 Нічний мікропілінг і сяйво Комплекс гліколевої, молочної та саліцилової кислот м’яко відлущує ороговілі клітини, вирівнює тон і текстуру, запобігаючи тьмяності.
+🌿 Ліпідне відновлення Олії жожоба та ши поповнюють дефіцит власних ліпідів, роблячи шкіру оксамитовою та насиченою до ранку.
+💧 Тривала гідратація (PatcH2O™) Молекулярна сітка з гіалуронової кислоти, сечовини та трегалози утримує вологу всередині клітин протягом усього циклу сну.
+🍃 Вітамінний детокс і зміцнення Вітаміни А та Е стимулюють клітинне оновлення, а екстракти хвоща, хмелю та розмарину знімають набряклість і зміцнюють судини.
+Кому підійде
+Для шкіри з втратою пружності, нерівним рельєфом та ознаками фотостаріння. Текстура насичена, але комфортна, швидко засвоюється протягом ночі.
+Результат
+Вранці обличчя виглядає підтягнутим і відпочилим
+Зникають дрібні зморшки
+Зміцнюється овал обличчя
+Відновлюється здоровий тургор
+Застосування
+Щодня ввечері наносити на очищене обличчя, шию та зону декольте. Для посилення ефекту використовувати разом із сироваткою. Ідеально поєднується з денним кремом Ultimate Lifting Recovery 43.
+Активні компоненти
+Пентапептид-35, протеїни сої, комплекс PatcH2O™, сквалан, олії ши, жожоба, примули, кави, пікуї та дині калаха, вітаміни А та Е, альфа-ліпоєва кислота, екстракти хмелю, розмарину, хвоща, хвої та лимона.
+Відчуття на шкірі
+Живлення, ніжне зволоження, шовковисто-оксамитовий ефект.
+Текстура
+Живильний крем, щільний, але легкий, швидко вбирається.
+Аромат
+Делікатна зелено-квіткова композиція з легким фруктовим відтінком.</t>
+  </si>
+  <si>
+    <t>AL44</t>
+  </si>
+  <si>
+    <t>Очищуюче молочко з трав'яними екстрактами Anna Logor Silky Herbal Cleanser (Art.401), 350 мл</t>
+  </si>
+  <si>
+    <t>✨ Anna Logor Silky Herbal Cleanser – ніжне очищення та шовковиста шкіра! ✨
+🌿 Чому варто обрати це молочко:
+💧 Делікатно видаляє макіяж, забруднення та надлишки себуму
+🌸 Забезпечує комплексний догляд завдяки трав’яним екстрактам
+🛡️ Вирівнює рельєф шкіри та нейтралізує відчуття стягнутості
+⚡ Глибоко зволожує та пом’якшує
+🌟 Допомагає розгладити дрібні зморшки та дарує омолоджувальний ефект
+💚 Результат – чиста, доглянута та сяюча шкіра без сухості!
+📌 Активні компоненти:
+🌱 Оливкова олія – живлення та захист
+🌸 Вітаміни А, Е та С – антиоксидантна дія та омолодження
+🌿 Екстракти розмарину, хвої, лимона, хмелю, хвоща польового – тонізація, регенерація та відновлення
+📌 Особливості продукту:
+Приємний аромат та ніжна текстура
+Добре піниться та легко змивається
+Зручний флакон із дозатором – економне використання
+📌 Спосіб застосування:
+Нанести молочко на зволожену шкіру обличчя.
+Розподілити легкими рухами.
+Змити теплою водою.
+Для максимального ефекту використати тонік Silky Herbal Toner Anna Logor.
+✔️ Характеристики продукту:
+Тип: Очищувальне молочко з трав’яними екстрактами
+Об’єм: 350 мл
+Вікова категорія: 16+
+Тип шкіри: Суха та нормальна
+Бренд: Anna Logor
+Країна виробництва: 🇺🇦 Україна
+🌟 Anna Logor Silky Herbal Cleanser – твій must-have для ніжного очищення та збереження молодості шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>AL401</t>
+  </si>
+  <si>
+    <t>Комплексний очищуючий гель Anna Logor Purifying Complex Cleanser (Art.301), 350 мл</t>
+  </si>
+  <si>
+    <t>✨ Anna Logor Purifying Complex Cleanser – ідеальний баланс для комбінованої шкіри! ✨
+🌿 Чому варто обрати цей гель:
+💧 Ефективно видаляє надлишки себуму та звужує пори
+🌸 Пом’якшує, глибоко зволожує та делікатно освітлює шкіру
+🛡️ Стимулює процеси клітинного відновлення
+⚡ Покращує структуру та колір обличчя
+🌟 Дарує природну матовість і відчуття свіжості
+💚 Результат – доглянута, чиста та сяюча шкіра без дискомфорту!
+📌 Активні компоненти:
+🌱 Екстракти водяного кресу, шавлії, лимона, лопуха та плюща – природне очищення та тонізація
+⚡ Гліколева, лимонна, яблучна та молочна кислоти – м’яке відлущування та регенерація
+📌 Спосіб застосування:
+Нанесіть достатню кількість гелю на зволожену шкіру обличчя.
+Розподіліть легкими рухами.
+Ретельно змийте теплою водою.
+Для закріплення ефекту використайте тонік Purifying Complex Toner Anna Logor.
+✔️ Особливості продукту:
+Приємний аромат
+Зручний флакон із дозатором
+Економне використання
+Об’єм: 350 мл · Art.301
+Вікова категорія: 16+
+Тип шкіри: комбінована
+🌟 Anna Logor Purifying Complex Cleanser – твій must-have для щоденного догляду за комбінованою шкірою! 🌟</t>
+  </si>
+  <si>
+    <t>AL301</t>
+  </si>
+  <si>
+    <t>Омолоджуючий зміцнюючий-зволожуючий денний крем Anna Logor Mezotherapy Firming Moisturizer (Art.521), 250 мл</t>
+  </si>
+  <si>
+    <t>✨ Mezotherapy Firming Moisturizer – професійний ліфтинг та зволоження щодня! ✨
+🌿 Чому варто обрати цей крем:
+💧 Натуральний склад – кераміди, масло ши, гіалуронова кислота, протеїни сої, екстракти хмелю та розмарину
+🌸 Боротьба зі зморшками – зменшує мімічні лінії, заломи та дрібні зморшки
+🛡️ Глибоке зволоження – нормалізує водний баланс, усуває сухість та чутливість
+⚡ Ліфтинг-ефект – підвищує пружність, робить овал обличчя чітким і виразним
+💚 Результат – підтягнута, сяюча та доглянута шкіра вже після кількох застосувань!
+📌 Активні компоненти:
+🌱 Кераміди – відновлення бар’єрних функцій
+🌸 Масло ши – живлення та пом’якшення
+💧 Гіалуронова кислота – інтенсивне зволоження
+🛡️ Протеїни сої – підвищення еластичності
+🌿 Екстракти хмелю та розмарину – антиоксидантна дія та тонізація
+✔️ Переваги продукту:
+Натуральна формула без шкідливих компонентів
+Професійний догляд у домашніх умовах
+Відчутний ефект ліфтингу та зволоження
+Підходить для щоденного використання
+🌟 Mezotherapy Firming Moisturizer – твій must-have для збереження молодості та краси шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>AL521</t>
+  </si>
+  <si>
+    <t>Живильний пептидний нічний крем Perfect Skin Peptide-Rich Cream (Art.54), 50 мл</t>
+  </si>
+  <si>
+    <t>Нічний крем з платиною та пептидами: Розкішна реновація вашої шкіри
+Цей нічний крем — справжня квінтесенція сучасної косметології, створена для бездоганного догляду за зрілою шкірою. Поки ви насолоджуєтеся сном, інноваційна формула на основі дорогоцінної платини та пептидів проводить глобальну «реновацію» клітин, повертаючи обличчю природну щільність, шовковисту гладкість та здорове внутрішнє сяйво.
+💎 Секрет ефективності: Як це працює?
+Платинове омолодження (Platinum Peptides): Ключовий актив (Acetyl Tetrapeptide-17) у синергії з частинками колоїдної платини діє як надпотужний клітинний регенератор. Платина гарантує максимальну стабільність пептиду, що дозволяє йому ефективно запускати синтез колагену та еластину — фундаментальних елементів молодості шкіри.
+Нічне мікрооновлення: Делікатний комплекс гліколевої, молочної та саліцилової кислот забезпечує м'яке, фізіологічне оновлення. Він усуває вікову гіперкератозність (огрубіння), вирівнює тон та готує шкіру до максимального засвоєння поживних речовин.
+Розумне зволоження PatcH2O™: Передова система на основі гіалуронової кислоти, трегалози та сечовини створює на шкірі захисну молекулярну мікросітку. Вона дозовано віддає вологу протягом усієї ночі, надійно запобігаючи ефекту «ранкової пом’ятості».
+Інтенсивний живильний коктейль: Розкішна база з олій примули вечірньої та жожоба глибоко насичує стоншену шкіру, реставрує її бар’єрні функції та миттєво усуває сухість.
+Тонус та антиоксидантний захист: Вітаміни молодості (А та Е) сприяють клітинному омолодженню, а екстракти хвоща, хмелю та сосни тонізують тканини і зміцнюють мікросудини.
+✨ Для кого створений цей крем?
+Ідеальний вибір для власниць зрілої шкіри (45+), яка потребує глибокого відновлення, інтенсивної корекції зморшок та ефективного усунення в’ялості.
+Ваш результат: Вже на ранок шкіра стає неймовірно м’якою, «наповненою» та пружною. За умови регулярного використання платинові пептиди забезпечують виражений ліфтинг-ефект: моделюється овал обличчя, а шкіра набуває того самого доглянутого, «дорогого» вигляду.
+🌸 Сенсорний досвід та характеристики
+Текстура: Живильна, щільна, але напрочуд легка — миттєво та комфортно вбирається.
+Відчуття на шкірі: Глибоке живлення, ніжне зволоження та розкішний шовковисто-оксамитовий фініш.
+Аромат: Вишуканий парфумований букет із витонченими квітково-пудровими мотивами.
+Активний склад: Пептидні комплекси (зокрема гептапептид-17), сквалан, гіалуронова та молочна кислоти, комплекс ПатчН2О™, цінні олії (ши, жожоба, примули, кави, дині калахарі, камелії), вітаміни А та Е, рослинні екстракти (хміль, розмарин, хвощ, хвоя, лимон).
+🌙 Ритуал краси (Застосування)
+Щовечора наносьте крем на попередньо очищену шкіру обличчя, шиї та зони декольте.
+Порада експерта: Для досягнення максимального омолоджувального ефекту використовуйте крем після нанесення сироватки. В якості денного догляду ідеальним доповненням стане крем Derma-Restructurant 53.</t>
+  </si>
+  <si>
+    <t>AL54</t>
+  </si>
+  <si>
+    <t>Пінний очищувач обличчя Anna Logor Foaming Facial Cleanser (Art.1003), 160 мл</t>
+  </si>
+  <si>
+    <t>160 мл</t>
+  </si>
+  <si>
+    <t>Anna Logor Foaming Facial Cleanser (150 мл, Art.1003)
+📌 Основні характеристики
+Тип засобу: Очищувальна пінка з помпою-піноутворювачем.
+Об'єм / Артикул: 150 мл / Art.1003.
+Вікова категорія: 18+ (без обмежень).
+Призначення: Для всіх типів шкіри, зокрема сухої, чутливої та тьмяної.
+🧪 Активні компоненти та їхня дія
+КомпонентДія на шкіруКомплекс AHA-кислот + ЛимонМ'яко відлущують змертвілі клітини, вирівнюють рельєф, вибілюють та освіжають тон.Гіалуронова кислотаГлибоко зволожує, запобігає втраті вологи та відчуттю стягнутості після вмивання.Екстракти хвоща, розмарину, хвої та хмелюНадають антисептичний ефект, дезінфікують, тонізують та сприяють детоксикації.
+💧 Спосіб застосування
+Нанесіть необхідну кількість пінки масажними круговими рухами на вологу шкіру обличчя та шиї (уникаючи ділянки навколо очей).
+Масажуйте до розчинення макіяжу та забруднень.
+Змийте великою кількістю теплої води.
+Завершіть процедуру тоніком Anna Logor для відновлення pH-балансу.
+💡 Примітка щодо використання: Оскільки засіб містить AHA-кислоти (навіть у м'якій концентрації), під час ранкового догляду рекомендовано додатково наносити сонцезахисний засіб (SPF), особливо для чутливої шкіри.</t>
+  </si>
+  <si>
+    <t>AL1003</t>
+  </si>
+  <si>
+    <t>Гідрогелева маска з ПДРН Miore Magic Wand PDRN Hydrogel Mask, 1 шт</t>
+  </si>
+  <si>
+    <t>1 шт</t>
+  </si>
+  <si>
+    <t>Miore Magic Wand PDRN Hydrogel Mask — це мультифункціональна гідрогелева маска з ПДРН, яка працює миттєво та має пролонговану дію від 3 до 5 днів.
+Зняти запалення після процедур чи за 20 хвилин підготувати шкіру до важливої події? Вона може все!
+Чому це фаворит косметологів та клієнтів:
+💧 Миттєвий SOS-ефект: швидко знімає почервоніння, набряки та гіперемію.
+✨ Ефект «вау-сяйва»: вирівнює тон, підвищує тургор і робить шкіру оксамитовою на дотик.
+🌿 Альтернатива ін'єкціям: при регулярному використанні дає результат, порівняний із біоревіталізацією та ботулінотерапією — без болю, синців і реабілітації.
+🛡️ Регенерація та захист: прискорює відновлення шкіри після пілінгів, лазера, ін'єкцій та чисток.
+Потужний склад для видимого результату:
+ПДРН (PDRN) — запускають глибинні процеси регенерації та омолодження клітин.
+Аргірелін (Argireline) — пептид із ботокс-ефектом, що м'яко розгладжує мімічні зморшки.
+Гіалуронова кислота + Бета-глюкан — забезпечують глибоке зволоження та зміцнюють захисний бар'єр.
+Комплекс із 12 рослинних екстрактів (алое, ромашка, розмарин, юзу, лаванда тощо) — чинять потужну протизапальну та заспокійливу дію.
+Універсальний засіб: підходить як для закриття професійних процедур у кабінеті косметолога, так і для домашнього догляду «на вихід» або підтримки салонного ефекту.</t>
+  </si>
+  <si>
+    <t>AL9001</t>
+  </si>
+  <si>
+    <t>Омолоджуюча сироватка з пептидами Perfect Skin Nutri-Peptide Serum (Art.55), 30 мл</t>
+  </si>
+  <si>
+    <t>✨ 55 Nutri-Peptide Serum – інтенсивна корекція вікових змін! ✨
+🌿 Чому варто обрати цю сироватку:
+💧 Створена спеціально для шкіри 35–45 років
+🌸 Синергетичний комплекс пептидів стимулює синтез колагену та еластину
+🛡️ Вирівнює мікрорельєф та покращує колір обличчя
+⚡ Забезпечує ліфтинг-ефект і моделює чіткіший овал
+🌟 Зменшує пігментацію та запобігає появі нових плям
+💚 Результат – пружна, сяюча та доглянута шкіра без ознак втоми!
+📌 Результати застосування:
+Ліфтинг та відновлення – підвищення тургору та пружності
+Корекція пігментації – зменшення вікових плям
+Ефект «м’якого фокусу» – миттєве маскування недосконалостей
+Захист та зволоження – протидія передчасному старінню
+📌 Активні компоненти:
+🌱 Тетрапептид-11, гептапептид-14, гептапептид-15 – стимуляція синтезу колагену
+🌸 Протеїни сої – підвищення еластичності
+🛡️ Альфа-ліпоєва кислота – антиоксидантний захист
+🌿 Екстракти хмелю, розмарину, хвоща, хвої та лимона – регенерація та тонізація
+📌 Спосіб застосування:
+Нанести кілька крапель на очищену шкіру обличчя, шиї та декольте.
+Легкими круговими рухами розподілити до повного поглинання.
+Використовувати як самостійний засіб, під крем або як базу під макіяж.
+✔️ Характеристики продукту:
+Тип: Омолоджувальна пептидна сироватка
+Об’єм: 30 мл
+Призначення: Проти зморшок, пігментації, сухості, ліфтинг
+Тип шкіри: Для всіх типів
+Вікова категорія: 35–45 років (35+)
+Клас косметики: Професійна
+Екотренди: Cruelty-free (не тестується на тваринах)
+Країна-виробник: 🇺🇸 США
+🌟 55 Nutri-Peptide Serum – твій must-have для інтенсивного омолодження та сяйва шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>AL55</t>
   </si>
 </sst>
 </file>
@@ -6122,7 +6605,79 @@
     <cellStyle name="Відсотковий" xfId="1" builtinId="5"/>
     <cellStyle name="Звичайний" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="33">
+  <dxfs count="42">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9EAD3"/>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9EAD3"/>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9EAD3"/>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -6647,7 +7202,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K166"/>
+  <dimension ref="A1:K240"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" style="9" customWidth="1"/>
@@ -11757,144 +12312,1262 @@
         <v>568</v>
       </c>
     </row>
-    <row r="161" spans="3:9" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A161" s="9" t="s">
+        <v>571</v>
+      </c>
+      <c r="B161" s="10" t="s">
+        <v>569</v>
+      </c>
       <c r="C161" s="10" t="s">
         <v>560</v>
       </c>
-      <c r="G161" s="2"/>
+      <c r="D161" s="10">
+        <v>850</v>
+      </c>
+      <c r="E161" s="10">
+        <v>560</v>
+      </c>
+      <c r="G161" s="2">
+        <v>11</v>
+      </c>
+      <c r="H161" s="10" t="s">
+        <v>558</v>
+      </c>
       <c r="I161" s="10" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="162" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="J161" s="10" t="s">
+        <v>570</v>
+      </c>
+      <c r="K161" s="9" t="s">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="162" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A162" s="9" t="s">
+        <v>575</v>
+      </c>
+      <c r="B162" s="10" t="s">
+        <v>572</v>
+      </c>
       <c r="C162" s="10" t="s">
         <v>560</v>
       </c>
-      <c r="G162" s="2"/>
+      <c r="D162" s="10">
+        <v>950</v>
+      </c>
+      <c r="E162" s="10">
+        <v>830</v>
+      </c>
+      <c r="G162" s="2">
+        <v>12</v>
+      </c>
+      <c r="H162" s="10" t="s">
+        <v>573</v>
+      </c>
       <c r="I162" s="10" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="163" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="J162" s="10" t="s">
+        <v>574</v>
+      </c>
+      <c r="K162" s="9" t="s">
+        <v>575</v>
+      </c>
+    </row>
+    <row r="163" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A163" s="9" t="s">
+        <v>578</v>
+      </c>
+      <c r="B163" s="10" t="s">
+        <v>576</v>
+      </c>
       <c r="C163" s="10" t="s">
         <v>560</v>
       </c>
-      <c r="G163" s="2"/>
+      <c r="D163" s="10">
+        <v>730</v>
+      </c>
+      <c r="E163" s="10">
+        <v>500</v>
+      </c>
+      <c r="G163" s="2">
+        <v>23</v>
+      </c>
+      <c r="H163" s="10" t="s">
+        <v>558</v>
+      </c>
       <c r="I163" s="10" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="164" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="J163" s="10" t="s">
+        <v>577</v>
+      </c>
+      <c r="K163" s="9" t="s">
+        <v>578</v>
+      </c>
+    </row>
+    <row r="164" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A164" s="9" t="s">
+        <v>582</v>
+      </c>
+      <c r="B164" s="10" t="s">
+        <v>579</v>
+      </c>
       <c r="C164" s="10" t="s">
         <v>560</v>
       </c>
-      <c r="G164" s="2"/>
+      <c r="D164" s="10">
+        <v>1350</v>
+      </c>
+      <c r="E164" s="10">
+        <v>1070</v>
+      </c>
+      <c r="G164" s="2">
+        <v>12</v>
+      </c>
+      <c r="H164" s="10" t="s">
+        <v>580</v>
+      </c>
       <c r="I164" s="10" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="165" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="J164" s="10" t="s">
+        <v>581</v>
+      </c>
+      <c r="K164" s="9" t="s">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="165" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A165" s="9" t="s">
+        <v>585</v>
+      </c>
+      <c r="B165" s="10" t="s">
+        <v>583</v>
+      </c>
       <c r="C165" s="10" t="s">
         <v>560</v>
       </c>
-      <c r="G165" s="2"/>
-    </row>
-    <row r="166" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="D165" s="10">
+        <v>790</v>
+      </c>
+      <c r="E165" s="10">
+        <v>570</v>
+      </c>
+      <c r="G165" s="2">
+        <v>12</v>
+      </c>
+      <c r="H165" s="10" t="s">
+        <v>558</v>
+      </c>
+      <c r="I165" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="J165" s="10" t="s">
+        <v>584</v>
+      </c>
+      <c r="K165" s="9" t="s">
+        <v>585</v>
+      </c>
+    </row>
+    <row r="166" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A166" s="9" t="s">
+        <v>588</v>
+      </c>
+      <c r="B166" s="10" t="s">
+        <v>586</v>
+      </c>
       <c r="C166" s="10" t="s">
         <v>560</v>
+      </c>
+      <c r="D166" s="10">
+        <v>1700</v>
+      </c>
+      <c r="E166" s="10">
+        <v>1430</v>
+      </c>
+      <c r="G166" s="2">
+        <v>21</v>
+      </c>
+      <c r="H166" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="I166" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="J166" s="10" t="s">
+        <v>587</v>
+      </c>
+      <c r="K166" s="9" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="167" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A167" s="9" t="s">
+        <v>591</v>
+      </c>
+      <c r="B167" s="10" t="s">
+        <v>589</v>
+      </c>
+      <c r="C167" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="D167" s="10">
+        <v>1100</v>
+      </c>
+      <c r="E167" s="10">
+        <v>830</v>
+      </c>
+      <c r="G167" s="2">
+        <v>26</v>
+      </c>
+      <c r="H167" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="I167" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="J167" s="10" t="s">
+        <v>590</v>
+      </c>
+      <c r="K167" s="9" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="168" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A168" s="9" t="s">
+        <v>594</v>
+      </c>
+      <c r="B168" s="10" t="s">
+        <v>592</v>
+      </c>
+      <c r="C168" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="D168" s="10">
+        <v>1800</v>
+      </c>
+      <c r="E168" s="10">
+        <v>1510</v>
+      </c>
+      <c r="G168" s="2">
+        <v>23</v>
+      </c>
+      <c r="H168" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="I168" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="J168" s="10" t="s">
+        <v>593</v>
+      </c>
+      <c r="K168" s="9" t="s">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="169" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A169" s="9" t="s">
+        <v>597</v>
+      </c>
+      <c r="B169" s="10" t="s">
+        <v>595</v>
+      </c>
+      <c r="C169" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="D169" s="10">
+        <v>750</v>
+      </c>
+      <c r="E169" s="10">
+        <v>590</v>
+      </c>
+      <c r="G169" s="2">
+        <v>22</v>
+      </c>
+      <c r="H169" s="10" t="s">
+        <v>558</v>
+      </c>
+      <c r="I169" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="J169" s="10" t="s">
+        <v>596</v>
+      </c>
+      <c r="K169" s="9" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="170" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A170" s="9" t="s">
+        <v>600</v>
+      </c>
+      <c r="B170" s="10" t="s">
+        <v>598</v>
+      </c>
+      <c r="C170" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="D170" s="10">
+        <v>800</v>
+      </c>
+      <c r="E170" s="10">
+        <v>560</v>
+      </c>
+      <c r="G170" s="2">
+        <v>17</v>
+      </c>
+      <c r="H170" s="10" t="s">
+        <v>558</v>
+      </c>
+      <c r="I170" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="J170" s="10" t="s">
+        <v>599</v>
+      </c>
+      <c r="K170" s="9" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="171" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A171" s="9" t="s">
+        <v>603</v>
+      </c>
+      <c r="B171" s="10" t="s">
+        <v>601</v>
+      </c>
+      <c r="C171" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="D171" s="10">
+        <v>2100</v>
+      </c>
+      <c r="E171" s="10">
+        <v>1700</v>
+      </c>
+      <c r="G171" s="2">
+        <v>21</v>
+      </c>
+      <c r="H171" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="I171" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="J171" s="10" t="s">
+        <v>602</v>
+      </c>
+      <c r="K171" s="9" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="172" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A172" s="9" t="s">
+        <v>606</v>
+      </c>
+      <c r="B172" s="10" t="s">
+        <v>604</v>
+      </c>
+      <c r="C172" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="D172" s="10">
+        <v>1900</v>
+      </c>
+      <c r="E172" s="10">
+        <v>1670</v>
+      </c>
+      <c r="G172" s="2">
+        <v>25</v>
+      </c>
+      <c r="H172" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="I172" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="J172" s="10" t="s">
+        <v>605</v>
+      </c>
+      <c r="K172" s="9" t="s">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="173" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A173" s="9" t="s">
+        <v>610</v>
+      </c>
+      <c r="B173" s="10" t="s">
+        <v>607</v>
+      </c>
+      <c r="C173" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="D173" s="10">
+        <v>730</v>
+      </c>
+      <c r="E173" s="10">
+        <v>540</v>
+      </c>
+      <c r="G173" s="2">
+        <v>15</v>
+      </c>
+      <c r="H173" s="10" t="s">
+        <v>608</v>
+      </c>
+      <c r="I173" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="J173" s="10" t="s">
+        <v>609</v>
+      </c>
+      <c r="K173" s="9" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="174" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A174" s="9" t="s">
+        <v>614</v>
+      </c>
+      <c r="B174" s="10" t="s">
+        <v>611</v>
+      </c>
+      <c r="C174" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="D174" s="10">
+        <v>600</v>
+      </c>
+      <c r="E174" s="10">
+        <v>420</v>
+      </c>
+      <c r="G174" s="2">
+        <v>18</v>
+      </c>
+      <c r="H174" s="10" t="s">
+        <v>612</v>
+      </c>
+      <c r="I174" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="J174" s="10" t="s">
+        <v>613</v>
+      </c>
+      <c r="K174" s="9" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="175" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A175" s="9" t="s">
+        <v>617</v>
+      </c>
+      <c r="B175" s="10" t="s">
+        <v>615</v>
+      </c>
+      <c r="C175" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="D175" s="10">
+        <v>1800</v>
+      </c>
+      <c r="E175" s="10">
+        <v>1500</v>
+      </c>
+      <c r="G175" s="2">
+        <v>21</v>
+      </c>
+      <c r="H175" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="I175" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="J175" s="10" t="s">
+        <v>616</v>
+      </c>
+      <c r="K175" s="9" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="176" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="C176" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G176" s="2"/>
+      <c r="I176" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="177" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C177" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G177" s="2"/>
+      <c r="I177" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="178" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C178" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G178" s="2"/>
+      <c r="I178" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="179" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C179" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G179" s="2"/>
+      <c r="I179" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="180" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C180" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G180" s="2"/>
+      <c r="I180" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="181" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C181" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G181" s="2"/>
+      <c r="I181" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="182" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C182" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G182" s="2"/>
+      <c r="I182" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="183" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C183" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G183" s="2"/>
+      <c r="I183" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="184" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C184" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G184" s="2"/>
+      <c r="I184" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="185" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C185" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G185" s="2"/>
+      <c r="I185" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="186" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C186" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G186" s="2"/>
+      <c r="I186" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="187" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C187" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G187" s="2"/>
+      <c r="I187" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="188" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C188" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G188" s="2"/>
+      <c r="I188" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="189" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C189" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G189" s="2"/>
+      <c r="I189" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="190" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C190" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G190" s="2"/>
+      <c r="I190" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="191" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C191" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G191" s="2"/>
+      <c r="I191" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="192" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C192" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G192" s="2"/>
+      <c r="I192" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="193" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C193" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G193" s="2"/>
+      <c r="I193" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="194" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C194" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G194" s="2"/>
+      <c r="I194" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="195" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C195" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G195" s="2"/>
+      <c r="I195" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="196" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C196" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G196" s="2"/>
+      <c r="I196" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="197" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C197" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G197" s="2"/>
+      <c r="I197" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="198" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C198" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G198" s="2"/>
+      <c r="I198" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="199" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C199" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G199" s="2"/>
+      <c r="I199" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="200" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C200" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G200" s="2"/>
+      <c r="I200" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="201" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C201" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G201" s="2"/>
+      <c r="I201" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="202" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C202" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G202" s="2"/>
+      <c r="I202" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="203" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C203" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G203" s="2"/>
+      <c r="I203" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="204" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C204" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G204" s="2"/>
+      <c r="I204" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="205" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C205" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G205" s="2"/>
+      <c r="I205" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="206" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C206" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G206" s="2"/>
+      <c r="I206" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="207" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C207" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G207" s="2"/>
+      <c r="I207" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="208" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C208" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G208" s="2"/>
+      <c r="I208" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="209" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C209" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G209" s="2"/>
+      <c r="I209" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="210" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C210" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="G210" s="2"/>
+      <c r="I210" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="211" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C211" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="I211" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="212" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C212" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="I212" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="213" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C213" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="I213" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="214" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C214" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="I214" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="215" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="C215" s="10" t="s">
+        <v>560</v>
+      </c>
+      <c r="I215" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="216" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="I216" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="217" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="I217" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="218" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="I218" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="219" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="I219" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="220" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="I220" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="221" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="I221" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="222" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="I222" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="223" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="I223" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="224" spans="3:9" x14ac:dyDescent="0.3">
+      <c r="I224" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="225" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I225" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="226" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I226" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="227" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I227" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="228" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I228" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="229" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I229" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="230" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I230" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="231" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I231" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="232" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I232" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="233" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I233" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="234" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I234" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="235" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I235" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="236" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I236" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="237" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I237" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="238" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I238" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="239" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I239" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="240" spans="9:9" x14ac:dyDescent="0.3">
+      <c r="I240" s="10" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K93" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="G2:G93">
-    <cfRule type="cellIs" dxfId="32" priority="31" operator="equal">
+    <cfRule type="cellIs" dxfId="41" priority="31" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="31" priority="32" operator="lessThan">
+    <cfRule type="cellIs" dxfId="40" priority="32" operator="lessThan">
       <formula>20</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="33" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="39" priority="33" operator="greaterThanOrEqual">
       <formula>20</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G94">
-    <cfRule type="cellIs" dxfId="29" priority="28" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="28" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="29" operator="lessThan">
+    <cfRule type="cellIs" dxfId="37" priority="29" operator="lessThan">
       <formula>20</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="30" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="36" priority="30" operator="greaterThanOrEqual">
       <formula>20</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G95">
-    <cfRule type="cellIs" dxfId="26" priority="25" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="25" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="25" priority="26" operator="lessThan">
+    <cfRule type="cellIs" dxfId="34" priority="26" operator="lessThan">
       <formula>20</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="27" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="33" priority="27" operator="greaterThanOrEqual">
       <formula>20</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G96">
-    <cfRule type="cellIs" dxfId="23" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="22" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="23" operator="lessThan">
+    <cfRule type="cellIs" dxfId="31" priority="23" operator="lessThan">
       <formula>20</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="24" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="30" priority="24" operator="greaterThanOrEqual">
       <formula>20</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G97">
-    <cfRule type="cellIs" dxfId="20" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="19" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="20" operator="lessThan">
+    <cfRule type="cellIs" dxfId="28" priority="20" operator="lessThan">
       <formula>20</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="21" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="27" priority="21" operator="greaterThanOrEqual">
       <formula>20</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G98">
-    <cfRule type="cellIs" dxfId="17" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="16" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="17" operator="lessThan">
+    <cfRule type="cellIs" dxfId="25" priority="17" operator="lessThan">
       <formula>20</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="15" priority="18" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="24" priority="18" operator="greaterThanOrEqual">
       <formula>20</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G99:G113">
-    <cfRule type="cellIs" dxfId="14" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="13" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="13" priority="14" operator="lessThan">
+    <cfRule type="cellIs" dxfId="22" priority="14" operator="lessThan">
       <formula>20</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="15" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="21" priority="15" operator="greaterThanOrEqual">
       <formula>20</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G114:G158">
-    <cfRule type="cellIs" dxfId="11" priority="10" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="10" operator="equal">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="11" operator="lessThan">
+    <cfRule type="cellIs" dxfId="19" priority="11" operator="lessThan">
       <formula>20</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="12" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="18" priority="12" operator="greaterThanOrEqual">
       <formula>20</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G159">
+    <cfRule type="cellIs" dxfId="17" priority="7" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="16" priority="8" operator="lessThan">
+      <formula>20</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="15" priority="9" operator="greaterThanOrEqual">
+      <formula>20</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G160">
+    <cfRule type="cellIs" dxfId="14" priority="4" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="13" priority="5" operator="lessThan">
+      <formula>20</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="6" operator="greaterThanOrEqual">
+      <formula>20</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G161:G210">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="lessThan">
+      <formula>20</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="3" operator="greaterThanOrEqual">
+      <formula>20</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E45EA910-30FA-4249-8083-D795408425A3}">
+  <dimension ref="A1:K5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" s="2">
+        <v>3500</v>
+      </c>
+      <c r="E2" s="2">
+        <v>3100</v>
+      </c>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2">
+        <v>10</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="K2" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="2">
+        <v>2420</v>
+      </c>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2">
+        <v>16</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="2">
+        <v>2800</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2">
+        <v>14</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="2">
+        <v>4100</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2">
+        <v>17</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>118</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="G2">
     <cfRule type="cellIs" dxfId="8" priority="7" operator="equal">
       <formula>0</formula>
     </cfRule>
@@ -11905,7 +13578,7 @@
       <formula>20</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G160">
+  <conditionalFormatting sqref="G3:G4">
     <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
       <formula>0</formula>
     </cfRule>
@@ -11916,7 +13589,7 @@
       <formula>20</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G161:G165">
+  <conditionalFormatting sqref="G5">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>0</formula>
     </cfRule>
@@ -11927,7 +13600,6 @@
       <formula>20</formula>
     </cfRule>
   </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>